<commit_message>
Bugle April 18, 2026
</commit_message>
<xml_diff>
--- a/Troop 79 Bugle Calendar for ICS Feed.xlsx
+++ b/Troop 79 Bugle Calendar for ICS Feed.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="798" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="804" uniqueCount="265">
   <si>
     <t>start_date</t>
   </si>
@@ -111,7 +111,7 @@
     <t>1b8d354bdf2aba78ef79bb44e04dde77@sheet2ics</t>
   </si>
   <si>
-    <t>Maya Eagle Project - I</t>
+    <t xml:space="preserve">Maya Eagle Project - I </t>
   </si>
   <si>
     <t>Repair Library and Sign</t>
@@ -150,6 +150,18 @@
     <t>8f47e9ac8233a825ca1e54ece63c20ca@sheet2ics</t>
   </si>
   <si>
+    <t>Maya Eagle Project - II</t>
+  </si>
+  <si>
+    <t>Install Library and Sign</t>
+  </si>
+  <si>
+    <t>Urban Ecology Center - 1500 E Park Place</t>
+  </si>
+  <si>
+    <t>a1d78be9122977477275ee0d478a7d78@sheet2ics</t>
+  </si>
+  <si>
     <t>Spring Campout - Meal Planning</t>
   </si>
   <si>
@@ -210,6 +222,72 @@
     <t>fa6dad6af2a3cec975ad87e08b6a2c2a@sheet2ics</t>
   </si>
   <si>
+    <t>No Troop Meeting</t>
+  </si>
+  <si>
+    <t>Memorial Day Weekend</t>
+  </si>
+  <si>
+    <t>31e16f14964d4a6bab2ba25f070774a4@sheet2ics</t>
+  </si>
+  <si>
+    <t>TBD</t>
+  </si>
+  <si>
+    <t>bc71eaf15abdc3a5673e8d6721de7f00@sheet2ics</t>
+  </si>
+  <si>
+    <t>849dd533a5088b786aa5d3d25ee9b681@sheet2ics</t>
+  </si>
+  <si>
+    <t>Prepare for High Adventure Trip</t>
+  </si>
+  <si>
+    <t>7222db9d6348d0631faa2378d1c8ee88@sheet2ics</t>
+  </si>
+  <si>
+    <t>High Adventure Trip</t>
+  </si>
+  <si>
+    <t>BWCA</t>
+  </si>
+  <si>
+    <t>02e52d7fe6a30e4623930f66937f1701@sheet2ics</t>
+  </si>
+  <si>
+    <t>05ea088280e099fce97694e4f6ddf12f@sheet2ics</t>
+  </si>
+  <si>
+    <t>Camp Physicals</t>
+  </si>
+  <si>
+    <t>107491addb3b9576ed2b5be31a06f102@sheet2ics</t>
+  </si>
+  <si>
+    <t>Fourth of July</t>
+  </si>
+  <si>
+    <t>290ab3dfb24f23c44b85ee236bcbf1ee@sheet2ics</t>
+  </si>
+  <si>
+    <t>38b737926b25d932e994b62a7b15a29d@sheet2ics</t>
+  </si>
+  <si>
+    <t>0df89d505ff7db5d0fd6917fadcafbeb@sheet2ics</t>
+  </si>
+  <si>
+    <t>Summer Camp - Tesomas</t>
+  </si>
+  <si>
+    <t>Tesomas Scout Reservation</t>
+  </si>
+  <si>
+    <t>5403 Spider Lake Rd, Rhinelander, WI 54501</t>
+  </si>
+  <si>
+    <t>1b0cff4a338d00c5b8e27f8b9a02eac4@sheet2ics</t>
+  </si>
+  <si>
     <t>Rummage Sale</t>
   </si>
   <si>
@@ -220,72 +298,6 @@
   </si>
   <si>
     <t>2a356e920aad675a7efea5fc90141738@sheet2ics</t>
-  </si>
-  <si>
-    <t>No Troop Meeting</t>
-  </si>
-  <si>
-    <t>Memorial Day Weekend</t>
-  </si>
-  <si>
-    <t>31e16f14964d4a6bab2ba25f070774a4@sheet2ics</t>
-  </si>
-  <si>
-    <t>TBD</t>
-  </si>
-  <si>
-    <t>bc71eaf15abdc3a5673e8d6721de7f00@sheet2ics</t>
-  </si>
-  <si>
-    <t>849dd533a5088b786aa5d3d25ee9b681@sheet2ics</t>
-  </si>
-  <si>
-    <t>Prepare for High Adventure Trip</t>
-  </si>
-  <si>
-    <t>7222db9d6348d0631faa2378d1c8ee88@sheet2ics</t>
-  </si>
-  <si>
-    <t>High Adventure Trip</t>
-  </si>
-  <si>
-    <t>BWCA</t>
-  </si>
-  <si>
-    <t>02e52d7fe6a30e4623930f66937f1701@sheet2ics</t>
-  </si>
-  <si>
-    <t>05ea088280e099fce97694e4f6ddf12f@sheet2ics</t>
-  </si>
-  <si>
-    <t>Camp Physicals</t>
-  </si>
-  <si>
-    <t>107491addb3b9576ed2b5be31a06f102@sheet2ics</t>
-  </si>
-  <si>
-    <t>Fourth of July</t>
-  </si>
-  <si>
-    <t>290ab3dfb24f23c44b85ee236bcbf1ee@sheet2ics</t>
-  </si>
-  <si>
-    <t>38b737926b25d932e994b62a7b15a29d@sheet2ics</t>
-  </si>
-  <si>
-    <t>0df89d505ff7db5d0fd6917fadcafbeb@sheet2ics</t>
-  </si>
-  <si>
-    <t>Summer Camp - Tesomas</t>
-  </si>
-  <si>
-    <t>Tesomas Scout Reservation</t>
-  </si>
-  <si>
-    <t>5403 Spider Lake Rd, Rhinelander, WI 54501</t>
-  </si>
-  <si>
-    <t>1b0cff4a338d00c5b8e27f8b9a02eac4@sheet2ics</t>
   </si>
   <si>
     <t>Court of Honor</t>
@@ -1390,16 +1402,16 @@
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="2">
-        <v>46135.0</v>
+        <v>46134.0</v>
       </c>
       <c r="B7" s="3">
-        <v>0.7916666666678793</v>
+        <v>0.7291666666678793</v>
       </c>
       <c r="C7" s="2">
-        <v>46135.0</v>
+        <v>46134.0</v>
       </c>
       <c r="D7" s="4">
-        <v>0.875</v>
+        <v>0.8125</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>31</v>
@@ -1521,57 +1533,57 @@
         <v>46145.0</v>
       </c>
       <c r="B11" s="3">
-        <v>0.6666666666678793</v>
+        <v>0.4583333333321207</v>
       </c>
       <c r="C11" s="2">
         <v>46145.0</v>
       </c>
       <c r="D11" s="4">
-        <v>0.7291666666678793</v>
+        <v>0.5833333333321207</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="I11" s="5" t="s">
         <v>13</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="2">
-        <v>46149.0</v>
+        <v>46145.0</v>
       </c>
       <c r="B12" s="3">
-        <v>0.75</v>
+        <v>0.6666666666678793</v>
       </c>
       <c r="C12" s="2">
-        <v>46149.0</v>
-      </c>
-      <c r="D12" s="3">
-        <v>0.7916666666678793</v>
+        <v>46145.0</v>
+      </c>
+      <c r="D12" s="4">
+        <v>0.7291666666678793</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>46</v>
+        <v>12</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>48</v>
+        <v>17</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>46</v>
+        <v>12</v>
       </c>
       <c r="I12" s="5" t="s">
         <v>13</v>
@@ -1582,16 +1594,16 @@
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="2">
-        <v>46150.0</v>
+        <v>46149.0</v>
       </c>
       <c r="B13" s="3">
         <v>0.75</v>
       </c>
       <c r="C13" s="2">
-        <v>46152.0</v>
-      </c>
-      <c r="D13" s="4">
-        <v>0.5</v>
+        <v>46149.0</v>
+      </c>
+      <c r="D13" s="3">
+        <v>0.7916666666678793</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>50</v>
@@ -1599,75 +1611,75 @@
       <c r="F13" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="G13" s="6" t="s">
+      <c r="G13" s="5" t="s">
         <v>52</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="I13" s="5" t="s">
         <v>13</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="2">
-        <v>46152.0</v>
+        <v>46150.0</v>
       </c>
       <c r="B14" s="3">
-        <v>0.6666666666678793</v>
+        <v>0.75</v>
       </c>
       <c r="C14" s="2">
         <v>46152.0</v>
       </c>
       <c r="D14" s="4">
-        <v>0.7291666666678793</v>
+        <v>0.5</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>12</v>
+        <v>54</v>
       </c>
       <c r="F14" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="G14" s="5" t="s">
-        <v>17</v>
+      <c r="G14" s="6" t="s">
+        <v>56</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="I14" s="5" t="s">
         <v>13</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1">
       <c r="A15" s="2">
-        <v>46156.0</v>
+        <v>46152.0</v>
       </c>
       <c r="B15" s="3">
-        <v>0.75</v>
+        <v>0.6666666666678793</v>
       </c>
       <c r="C15" s="2">
-        <v>46156.0</v>
-      </c>
-      <c r="D15" s="3">
-        <v>0.2916666666678793</v>
+        <v>46152.0</v>
+      </c>
+      <c r="D15" s="4">
+        <v>0.7291666666678793</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>57</v>
+        <v>12</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>59</v>
+        <v>17</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>53</v>
+        <v>12</v>
       </c>
       <c r="I15" s="5" t="s">
         <v>13</v>
@@ -1678,16 +1690,16 @@
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="2">
-        <v>46157.0</v>
+        <v>46156.0</v>
       </c>
       <c r="B16" s="3">
         <v>0.75</v>
       </c>
       <c r="C16" s="2">
-        <v>46159.0</v>
+        <v>46156.0</v>
       </c>
       <c r="D16" s="3">
-        <v>0.5833333333321207</v>
+        <v>0.2916666666678793</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>61</v>
@@ -1696,42 +1708,42 @@
         <v>62</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="I16" s="5" t="s">
         <v>13</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="2">
-        <v>46165.0</v>
+        <v>46157.0</v>
       </c>
       <c r="B17" s="3">
-        <v>0.375</v>
+        <v>0.75</v>
       </c>
       <c r="C17" s="2">
-        <v>46165.0</v>
-      </c>
-      <c r="D17" s="4">
-        <v>0.75</v>
+        <v>46159.0</v>
+      </c>
+      <c r="D17" s="3">
+        <v>0.5833333333321207</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="I17" s="5" t="s">
         <v>13</v>
@@ -2077,7 +2089,7 @@
         <v>88</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="I28" s="5" t="s">
         <v>13</v>
@@ -2087,17 +2099,17 @@
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="7">
-        <v>46278.0</v>
-      </c>
-      <c r="B29" s="4">
-        <v>0.625</v>
-      </c>
-      <c r="C29" s="7">
-        <v>46278.0</v>
-      </c>
-      <c r="D29" s="3">
-        <v>0.7916666666678793</v>
+      <c r="A29" s="2">
+        <v>46263.0</v>
+      </c>
+      <c r="B29" s="3">
+        <v>0.375</v>
+      </c>
+      <c r="C29" s="2">
+        <v>46263.0</v>
+      </c>
+      <c r="D29" s="4">
+        <v>0.75</v>
       </c>
       <c r="E29" s="5" t="s">
         <v>90</v>
@@ -2106,10 +2118,10 @@
         <v>91</v>
       </c>
       <c r="G29" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H29" s="5" t="s">
         <v>92</v>
-      </c>
-      <c r="H29" s="5" t="s">
-        <v>12</v>
       </c>
       <c r="I29" s="5" t="s">
         <v>13</v>
@@ -2119,7 +2131,36 @@
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="I30" s="8"/>
+      <c r="A30" s="7">
+        <v>46278.0</v>
+      </c>
+      <c r="B30" s="4">
+        <v>0.625</v>
+      </c>
+      <c r="C30" s="7">
+        <v>46278.0</v>
+      </c>
+      <c r="D30" s="3">
+        <v>0.7916666666678793</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="G30" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="H30" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I30" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="J30" s="5" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="I31" s="8"/>
@@ -5025,10 +5066,10 @@
         <v>6</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>0</v>
@@ -5043,43 +5084,43 @@
         <v>3</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="T1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
@@ -5096,7 +5137,7 @@
         <v>11</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G2" s="5" t="b">
         <v>0</v>
@@ -5117,10 +5158,10 @@
         <v>12</v>
       </c>
       <c r="U2" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W2" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
@@ -5140,7 +5181,7 @@
         <v>17</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G3" s="5" t="b">
         <v>0</v>
@@ -5164,10 +5205,10 @@
         <v>12</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
@@ -5178,7 +5219,7 @@
         <v>13</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>25</v>
@@ -5187,7 +5228,7 @@
         <v>17</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G4" s="5" t="b">
         <v>0</v>
@@ -5211,10 +5252,10 @@
         <v>12</v>
       </c>
       <c r="U4" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W4" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
@@ -5234,7 +5275,7 @@
         <v>21</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G5" s="5" t="b">
         <v>0</v>
@@ -5258,13 +5299,13 @@
         <v>22</v>
       </c>
       <c r="U5" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="V5" s="10" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="W5" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
@@ -5275,7 +5316,7 @@
         <v>13</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>38</v>
@@ -5284,7 +5325,7 @@
         <v>17</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G6" s="5" t="b">
         <v>0</v>
@@ -5305,10 +5346,10 @@
         <v>12</v>
       </c>
       <c r="U6" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W6" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
@@ -5328,7 +5369,7 @@
         <v>42</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G7" s="5" t="b">
         <v>0</v>
@@ -5352,16 +5393,16 @@
         <v>22</v>
       </c>
       <c r="U7" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="V7" s="11"/>
       <c r="W7" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="5" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>13</v>
@@ -5370,13 +5411,13 @@
         <v>12</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G8" s="5" t="b">
         <v>0</v>
@@ -5400,30 +5441,30 @@
         <v>12</v>
       </c>
       <c r="U8" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W8" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="5" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G9" s="5" t="b">
         <v>0</v>
@@ -5444,18 +5485,18 @@
         <v>30.0</v>
       </c>
       <c r="T9" s="5" t="s">
-        <v>66</v>
+        <v>92</v>
       </c>
       <c r="U9" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W9" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="5" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>13</v>
@@ -5464,13 +5505,13 @@
         <v>12</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G10" s="5" t="b">
         <v>0</v>
@@ -5494,30 +5535,30 @@
         <v>12</v>
       </c>
       <c r="U10" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W10" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="5" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>71</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G11" s="5" t="b">
         <v>0</v>
@@ -5535,13 +5576,13 @@
         <v>0.5833333333321207</v>
       </c>
       <c r="T11" s="5" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="U11" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W11" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
@@ -5558,7 +5599,7 @@
         <v>69</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G12" s="5" t="b">
         <v>0</v>
@@ -5576,10 +5617,10 @@
         <v>0.6673611111109494</v>
       </c>
       <c r="U12" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W12" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
@@ -5599,7 +5640,7 @@
         <v>17</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G13" s="5" t="b">
         <v>0</v>
@@ -5623,10 +5664,10 @@
         <v>12</v>
       </c>
       <c r="U13" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W13" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
@@ -5646,7 +5687,7 @@
         <v>17</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G14" s="5" t="b">
         <v>0</v>
@@ -5670,10 +5711,10 @@
         <v>12</v>
       </c>
       <c r="U14" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W14" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1">
@@ -5693,7 +5734,7 @@
         <v>17</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G15" s="5" t="b">
         <v>0</v>
@@ -5717,10 +5758,10 @@
         <v>12</v>
       </c>
       <c r="U15" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W15" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
@@ -5740,7 +5781,7 @@
         <v>77</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G16" s="5" t="b">
         <v>0</v>
@@ -5764,10 +5805,10 @@
         <v>29</v>
       </c>
       <c r="U16" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W16" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
@@ -5787,7 +5828,7 @@
         <v>17</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G17" s="5" t="b">
         <v>0</v>
@@ -5811,10 +5852,10 @@
         <v>12</v>
       </c>
       <c r="U17" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W17" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
@@ -5834,7 +5875,7 @@
         <v>17</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G18" s="5" t="b">
         <v>0</v>
@@ -5858,10 +5899,10 @@
         <v>12</v>
       </c>
       <c r="U18" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W18" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="19" ht="15.75" customHeight="1">
@@ -5878,7 +5919,7 @@
         <v>82</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G19" s="5" t="b">
         <v>0</v>
@@ -5902,10 +5943,10 @@
         <v>12</v>
       </c>
       <c r="U19" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W19" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
@@ -5925,7 +5966,7 @@
         <v>17</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G20" s="5" t="b">
         <v>0</v>
@@ -5949,10 +5990,10 @@
         <v>12</v>
       </c>
       <c r="U20" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W20" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
@@ -5972,7 +6013,7 @@
         <v>17</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G21" s="5" t="b">
         <v>0</v>
@@ -5996,10 +6037,10 @@
         <v>12</v>
       </c>
       <c r="U21" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W21" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
@@ -6019,7 +6060,7 @@
         <v>88</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G22" s="5" t="b">
         <v>0</v>
@@ -6037,33 +6078,33 @@
         <v>0.5416666666678793</v>
       </c>
       <c r="T22" s="5" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="U22" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W22" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="5" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G23" s="5" t="b">
         <v>0</v>
@@ -6084,10 +6125,10 @@
         <v>12</v>
       </c>
       <c r="U23" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W23" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
@@ -10867,22 +10908,22 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G1" s="5" t="b">
         <v>0</v>
@@ -10900,33 +10941,33 @@
         <v>0.7708333333321207</v>
       </c>
       <c r="T1" s="5" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="U1" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W1" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G2" s="5" t="b">
         <v>0</v>
@@ -10944,33 +10985,33 @@
         <v>0.8125</v>
       </c>
       <c r="T2" s="5" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="U2" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W2" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G3" s="5" t="b">
         <v>0</v>
@@ -10991,30 +11032,30 @@
         <v>22</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G4" s="5" t="b">
         <v>0</v>
@@ -11033,33 +11074,33 @@
       </c>
       <c r="L4" s="2"/>
       <c r="T4" s="5" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="U4" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W4" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G5" s="5" t="b">
         <v>0</v>
@@ -11077,16 +11118,16 @@
         <v>0.8125</v>
       </c>
       <c r="T5" s="5" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="U5" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W5" s="5"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>13</v>
@@ -11095,13 +11136,13 @@
         <v>12</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G6" s="5" t="b">
         <v>0</v>
@@ -11125,30 +11166,30 @@
         <v>12</v>
       </c>
       <c r="U6" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W6" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G7" s="5" t="b">
         <v>0</v>
@@ -11169,30 +11210,30 @@
         <v>22</v>
       </c>
       <c r="U7" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W7" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G8" s="5" t="b">
         <v>0</v>
@@ -11213,18 +11254,18 @@
         <v>60.0</v>
       </c>
       <c r="T8" s="5" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="U8" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W8" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>13</v>
@@ -11233,13 +11274,13 @@
         <v>12</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G9" s="5" t="b">
         <v>0</v>
@@ -11263,15 +11304,15 @@
         <v>12</v>
       </c>
       <c r="U9" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W9" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>13</v>
@@ -11280,13 +11321,13 @@
         <v>12</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G10" s="5" t="b">
         <v>0</v>
@@ -11310,15 +11351,15 @@
         <v>12</v>
       </c>
       <c r="U10" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W10" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>13</v>
@@ -11327,13 +11368,13 @@
         <v>12</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G11" s="5" t="b">
         <v>0</v>
@@ -11357,30 +11398,30 @@
         <v>12</v>
       </c>
       <c r="U11" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W11" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G12" s="5" t="b">
         <v>0</v>
@@ -11398,18 +11439,18 @@
         <v>0.8125</v>
       </c>
       <c r="T12" s="5" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="U12" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W12" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>13</v>
@@ -11418,13 +11459,13 @@
         <v>12</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G13" s="5" t="b">
         <v>0</v>
@@ -11448,30 +11489,30 @@
         <v>12</v>
       </c>
       <c r="U13" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W13" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G14" s="5" t="b">
         <v>0</v>
@@ -11495,15 +11536,15 @@
         <v>12</v>
       </c>
       <c r="U14" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W14" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>13</v>
@@ -11512,10 +11553,10 @@
         <v>68</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G15" s="5" t="b">
         <v>0</v>
@@ -11533,15 +11574,15 @@
         <v>0.6673611111109494</v>
       </c>
       <c r="U15" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W15" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>13</v>
@@ -11550,10 +11591,10 @@
         <v>68</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G16" s="5" t="b">
         <v>0</v>
@@ -11571,15 +11612,15 @@
         <v>0.6673611111109494</v>
       </c>
       <c r="U16" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W16" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>13</v>
@@ -11588,13 +11629,13 @@
         <v>12</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G17" s="5" t="b">
         <v>0</v>
@@ -11618,30 +11659,30 @@
         <v>12</v>
       </c>
       <c r="U17" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W17" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G18" s="5" t="b">
         <v>0</v>
@@ -11662,33 +11703,33 @@
         <v>30.0</v>
       </c>
       <c r="T18" s="5" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="U18" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W18" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="E19" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G19" s="5" t="b">
         <v>0</v>
@@ -11709,18 +11750,18 @@
         <v>30.0</v>
       </c>
       <c r="T19" s="5" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="U19" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W19" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="B20" s="5" t="s">
         <v>13</v>
@@ -11729,10 +11770,10 @@
         <v>68</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G20" s="5" t="b">
         <v>0</v>
@@ -11750,15 +11791,15 @@
         <v>0.6673611111109494</v>
       </c>
       <c r="U20" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W20" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>13</v>
@@ -11773,7 +11814,7 @@
         <v>17</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G21" s="5" t="b">
         <v>0</v>
@@ -11797,15 +11838,15 @@
         <v>12</v>
       </c>
       <c r="U21" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W21" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>13</v>
@@ -11820,7 +11861,7 @@
         <v>17</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G22" s="5" t="b">
         <v>0</v>
@@ -11844,30 +11885,30 @@
         <v>12</v>
       </c>
       <c r="U22" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W22" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="5" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="E23" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G23" s="5" t="b">
         <v>0</v>
@@ -11891,30 +11932,30 @@
         <v>12</v>
       </c>
       <c r="U23" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W23" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="5" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="E24" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G24" s="5" t="b">
         <v>0</v>
@@ -11938,30 +11979,30 @@
         <v>12</v>
       </c>
       <c r="U24" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W24" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="5" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="E25" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G25" s="5" t="b">
         <v>0</v>
@@ -11985,30 +12026,30 @@
         <v>12</v>
       </c>
       <c r="U25" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W25" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="5" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G26" s="5" t="b">
         <v>0</v>
@@ -12026,36 +12067,36 @@
         <v>0.6875</v>
       </c>
       <c r="T26" s="5" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="U26" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="V26" s="12" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="W26" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="5" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="E27" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G27" s="5" t="b">
         <v>0</v>
@@ -12073,31 +12114,31 @@
         <v>0.8125</v>
       </c>
       <c r="T27" s="5" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="U27" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W27" s="5"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="5" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="E28" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G28" s="5" t="b">
         <v>0</v>
@@ -12115,30 +12156,30 @@
         <v>0.6736111111094942</v>
       </c>
       <c r="U28" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W28" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="5" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G29" s="5" t="b">
         <v>0</v>
@@ -12156,33 +12197,33 @@
         <v>0.8125</v>
       </c>
       <c r="T29" s="5" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="U29" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W29" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="5" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G30" s="5" t="b">
         <v>0</v>
@@ -12206,30 +12247,30 @@
         <v>12</v>
       </c>
       <c r="U30" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W30" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="5" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="E31" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G31" s="5" t="b">
         <v>0</v>
@@ -12253,21 +12294,21 @@
         <v>22</v>
       </c>
       <c r="U31" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W31" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="5" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>16</v>
@@ -12276,7 +12317,7 @@
         <v>17</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G32" s="5" t="b">
         <v>0</v>
@@ -12300,30 +12341,30 @@
         <v>12</v>
       </c>
       <c r="U32" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W32" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="5" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G33" s="5" t="b">
         <v>0</v>
@@ -12341,24 +12382,24 @@
         <v>0.3958333333321207</v>
       </c>
       <c r="T33" s="5" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="U33" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W33" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="5" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>16</v>
@@ -12367,7 +12408,7 @@
         <v>17</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G34" s="5" t="b">
         <v>0</v>
@@ -12391,30 +12432,30 @@
         <v>12</v>
       </c>
       <c r="U34" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W34" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="5" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="B35" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="E35" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G35" s="5" t="b">
         <v>0</v>
@@ -12435,24 +12476,24 @@
         <v>30.0</v>
       </c>
       <c r="T35" s="5" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="U35" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W35" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="5" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="B36" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>16</v>
@@ -12461,7 +12502,7 @@
         <v>17</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G36" s="5" t="b">
         <v>0</v>
@@ -12485,30 +12526,30 @@
         <v>12</v>
       </c>
       <c r="U36" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W36" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="5" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="B37" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="E37" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G37" s="5" t="b">
         <v>0</v>
@@ -12526,28 +12567,28 @@
         <v>0.8125</v>
       </c>
       <c r="T37" s="5" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="U37" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W37" s="5"/>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="5" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="B38" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="F38" s="5"/>
       <c r="G38" s="5" t="b">
@@ -12569,21 +12610,21 @@
         <v>22</v>
       </c>
       <c r="U38" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W38" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="5" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>16</v>
@@ -12592,7 +12633,7 @@
         <v>17</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G39" s="5" t="b">
         <v>0</v>
@@ -12616,30 +12657,30 @@
         <v>12</v>
       </c>
       <c r="U39" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W39" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="5" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="B40" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="E40" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G40" s="5" t="b">
         <v>0</v>
@@ -12663,27 +12704,27 @@
         <v>12</v>
       </c>
       <c r="U40" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W40" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="5" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="B41" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G41" s="5" t="b">
         <v>0</v>
@@ -12704,10 +12745,10 @@
         <v>12</v>
       </c>
       <c r="U41" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="W41" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -12741,227 +12782,227 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="M1" s="13" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="M2" s="14" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
     </row>
     <row r="5">
       <c r="M5" s="15" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="M20" s="5" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="8" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="8" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="8" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="8" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="8" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="8" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="8" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1"/>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="8" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="8" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="8" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="8" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="8" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="8" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="8" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1"/>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="8" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="8" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="8" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="8" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1"/>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="8" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="8" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="8" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="8" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="8" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="8" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
Bugle May 31, 2026
</commit_message>
<xml_diff>
--- a/Troop 79 Bugle Calendar for ICS Feed.xlsx
+++ b/Troop 79 Bugle Calendar for ICS Feed.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="810" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="810" uniqueCount="272">
   <si>
     <t>start_date</t>
   </si>
@@ -231,163 +231,172 @@
     <t>31e16f14964d4a6bab2ba25f070774a4@sheet2ics</t>
   </si>
   <si>
+    <t>Campout Cleanup - MB and Rank Catchup</t>
+  </si>
+  <si>
+    <t>bc71eaf15abdc3a5673e8d6721de7f00@sheet2ics</t>
+  </si>
+  <si>
+    <t>Woodwork MB - Makeup / Finishup</t>
+  </si>
+  <si>
+    <t>849dd533a5088b786aa5d3d25ee9b681@sheet2ics</t>
+  </si>
+  <si>
+    <t>Prepare for High Adventure Trip</t>
+  </si>
+  <si>
+    <t>7222db9d6348d0631faa2378d1c8ee88@sheet2ics</t>
+  </si>
+  <si>
+    <t>High Adventure Trip</t>
+  </si>
+  <si>
+    <t>BWCA</t>
+  </si>
+  <si>
+    <t>02e52d7fe6a30e4623930f66937f1701@sheet2ics</t>
+  </si>
+  <si>
+    <t>05ea088280e099fce97694e4f6ddf12f@sheet2ics</t>
+  </si>
+  <si>
+    <t>Camp Physicals</t>
+  </si>
+  <si>
+    <t>107491addb3b9576ed2b5be31a06f102@sheet2ics</t>
+  </si>
+  <si>
+    <t>Fourth of July</t>
+  </si>
+  <si>
+    <t>290ab3dfb24f23c44b85ee236bcbf1ee@sheet2ics</t>
+  </si>
+  <si>
+    <t>Prep for Summer Camp</t>
+  </si>
+  <si>
+    <t>38b737926b25d932e994b62a7b15a29d@sheet2ics</t>
+  </si>
+  <si>
+    <t>0df89d505ff7db5d0fd6917fadcafbeb@sheet2ics</t>
+  </si>
+  <si>
+    <t>Summer Camp - Tesomas</t>
+  </si>
+  <si>
+    <t>Tesomas Scout Reservation</t>
+  </si>
+  <si>
+    <t>5403 Spider Lake Rd, Rhinelander, WI 54501</t>
+  </si>
+  <si>
+    <t>1b0cff4a338d00c5b8e27f8b9a02eac4@sheet2ics</t>
+  </si>
+  <si>
+    <t>Rummage Sale</t>
+  </si>
+  <si>
+    <t>All Day Rummage Sale</t>
+  </si>
+  <si>
+    <t>Fund Raiser</t>
+  </si>
+  <si>
+    <t>2a356e920aad675a7efea5fc90141738@sheet2ics</t>
+  </si>
+  <si>
+    <t>Court of Honor</t>
+  </si>
+  <si>
+    <t>Grant Park Picnic Area</t>
+  </si>
+  <si>
+    <t>Grant Park Picnic Area with Shelter</t>
+  </si>
+  <si>
+    <t>11a5cb096a7f6578a8ef2d5ed2b76687@sheet2ics</t>
+  </si>
+  <si>
+    <t>timezone</t>
+  </si>
+  <si>
+    <t>all_day</t>
+  </si>
+  <si>
+    <t>due_date</t>
+  </si>
+  <si>
+    <t>due_time</t>
+  </si>
+  <si>
+    <t>recurrence_rule</t>
+  </si>
+  <si>
+    <t>recurrence_until</t>
+  </si>
+  <si>
+    <t>recurrence_count</t>
+  </si>
+  <si>
+    <t>exdates</t>
+  </si>
+  <si>
+    <t>alarm_minutes_before</t>
+  </si>
+  <si>
+    <t>attendees</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>url</t>
+  </si>
+  <si>
+    <t>organizer_email</t>
+  </si>
+  <si>
+    <t>notes_internal</t>
+  </si>
+  <si>
+    <t>America/Chicago</t>
+  </si>
+  <si>
+    <t>CONFIRMED</t>
+  </si>
+  <si>
+    <t>bsatroop79bg@gmail.com</t>
+  </si>
+  <si>
+    <t>Troop Meeting - Wood Working MB</t>
+  </si>
+  <si>
+    <t>https://band.us/band/93239709/schedule/4%2F93239709%2F961498689%2F19700101</t>
+  </si>
+  <si>
+    <t>8f47e9ac8233a825ca1e54ece63c20ca@sheet2ics</t>
+  </si>
+  <si>
+    <t>Service Project - Oakleaf Trail Cleanup</t>
+  </si>
+  <si>
+    <t>Oakleaf Trail Cleanup</t>
+  </si>
+  <si>
+    <t>Colectivo Lakefront</t>
+  </si>
+  <si>
+    <t>b488cfbac2b9a8a809c579b888ed61ee@sheet2ics</t>
+  </si>
+  <si>
+    <t>Pancake Breakfast Fund Raiser</t>
+  </si>
+  <si>
+    <t>Annual Pancake Breakfast</t>
+  </si>
+  <si>
     <t>TBD</t>
-  </si>
-  <si>
-    <t>bc71eaf15abdc3a5673e8d6721de7f00@sheet2ics</t>
-  </si>
-  <si>
-    <t>849dd533a5088b786aa5d3d25ee9b681@sheet2ics</t>
-  </si>
-  <si>
-    <t>Prepare for High Adventure Trip</t>
-  </si>
-  <si>
-    <t>7222db9d6348d0631faa2378d1c8ee88@sheet2ics</t>
-  </si>
-  <si>
-    <t>High Adventure Trip</t>
-  </si>
-  <si>
-    <t>BWCA</t>
-  </si>
-  <si>
-    <t>02e52d7fe6a30e4623930f66937f1701@sheet2ics</t>
-  </si>
-  <si>
-    <t>05ea088280e099fce97694e4f6ddf12f@sheet2ics</t>
-  </si>
-  <si>
-    <t>Camp Physicals</t>
-  </si>
-  <si>
-    <t>107491addb3b9576ed2b5be31a06f102@sheet2ics</t>
-  </si>
-  <si>
-    <t>Fourth of July</t>
-  </si>
-  <si>
-    <t>290ab3dfb24f23c44b85ee236bcbf1ee@sheet2ics</t>
-  </si>
-  <si>
-    <t>38b737926b25d932e994b62a7b15a29d@sheet2ics</t>
-  </si>
-  <si>
-    <t>0df89d505ff7db5d0fd6917fadcafbeb@sheet2ics</t>
-  </si>
-  <si>
-    <t>Summer Camp - Tesomas</t>
-  </si>
-  <si>
-    <t>Tesomas Scout Reservation</t>
-  </si>
-  <si>
-    <t>5403 Spider Lake Rd, Rhinelander, WI 54501</t>
-  </si>
-  <si>
-    <t>1b0cff4a338d00c5b8e27f8b9a02eac4@sheet2ics</t>
-  </si>
-  <si>
-    <t>Rummage Sale</t>
-  </si>
-  <si>
-    <t>All Day Rummage Sale</t>
-  </si>
-  <si>
-    <t>Fund Raiser</t>
-  </si>
-  <si>
-    <t>2a356e920aad675a7efea5fc90141738@sheet2ics</t>
-  </si>
-  <si>
-    <t>Court of Honor</t>
-  </si>
-  <si>
-    <t>Grant Park Picnic Area</t>
-  </si>
-  <si>
-    <t>Grant Park Picnic Area with Shelter</t>
-  </si>
-  <si>
-    <t>11a5cb096a7f6578a8ef2d5ed2b76687@sheet2ics</t>
-  </si>
-  <si>
-    <t>timezone</t>
-  </si>
-  <si>
-    <t>all_day</t>
-  </si>
-  <si>
-    <t>due_date</t>
-  </si>
-  <si>
-    <t>due_time</t>
-  </si>
-  <si>
-    <t>recurrence_rule</t>
-  </si>
-  <si>
-    <t>recurrence_until</t>
-  </si>
-  <si>
-    <t>recurrence_count</t>
-  </si>
-  <si>
-    <t>exdates</t>
-  </si>
-  <si>
-    <t>alarm_minutes_before</t>
-  </si>
-  <si>
-    <t>attendees</t>
-  </si>
-  <si>
-    <t>status</t>
-  </si>
-  <si>
-    <t>url</t>
-  </si>
-  <si>
-    <t>organizer_email</t>
-  </si>
-  <si>
-    <t>notes_internal</t>
-  </si>
-  <si>
-    <t>America/Chicago</t>
-  </si>
-  <si>
-    <t>CONFIRMED</t>
-  </si>
-  <si>
-    <t>bsatroop79bg@gmail.com</t>
-  </si>
-  <si>
-    <t>Troop Meeting - Wood Working MB</t>
-  </si>
-  <si>
-    <t>https://band.us/band/93239709/schedule/4%2F93239709%2F961498689%2F19700101</t>
-  </si>
-  <si>
-    <t>8f47e9ac8233a825ca1e54ece63c20ca@sheet2ics</t>
-  </si>
-  <si>
-    <t>Service Project - Oakleaf Trail Cleanup</t>
-  </si>
-  <si>
-    <t>Oakleaf Trail Cleanup</t>
-  </si>
-  <si>
-    <t>Colectivo Lakefront</t>
-  </si>
-  <si>
-    <t>b488cfbac2b9a8a809c579b888ed61ee@sheet2ics</t>
-  </si>
-  <si>
-    <t>Pancake Breakfast Fund Raiser</t>
-  </si>
-  <si>
-    <t>Annual Pancake Breakfast</t>
   </si>
   <si>
     <t>8ab1c36a61c104dc8f881142028eb1b5@sheet2ics</t>
@@ -1842,7 +1851,7 @@
         <v>12</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G20" s="5" t="s">
         <v>17</v>
@@ -1854,7 +1863,7 @@
         <v>13</v>
       </c>
       <c r="J20" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
@@ -1874,7 +1883,7 @@
         <v>12</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G21" s="5" t="s">
         <v>17</v>
@@ -1886,7 +1895,7 @@
         <v>13</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
@@ -1903,13 +1912,13 @@
         <v>0.625</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H22" s="5" t="s">
         <v>29</v>
@@ -1918,7 +1927,7 @@
         <v>13</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
@@ -1938,7 +1947,7 @@
         <v>68</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G23" s="5" t="s">
         <v>17</v>
@@ -1950,7 +1959,7 @@
         <v>13</v>
       </c>
       <c r="J23" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
@@ -1970,7 +1979,7 @@
         <v>12</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G24" s="5" t="s">
         <v>17</v>
@@ -1982,7 +1991,7 @@
         <v>13</v>
       </c>
       <c r="J24" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
@@ -2002,7 +2011,7 @@
         <v>68</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="H25" s="5" t="s">
         <v>12</v>
@@ -2011,7 +2020,7 @@
         <v>13</v>
       </c>
       <c r="J25" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
@@ -2031,7 +2040,7 @@
         <v>12</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="G26" s="5" t="s">
         <v>17</v>
@@ -2043,7 +2052,7 @@
         <v>13</v>
       </c>
       <c r="J26" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
@@ -2063,7 +2072,7 @@
         <v>12</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="G27" s="5" t="s">
         <v>17</v>
@@ -2075,7 +2084,7 @@
         <v>13</v>
       </c>
       <c r="J27" s="5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
@@ -2092,13 +2101,13 @@
         <v>0.5416666666678793</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="H28" s="5" t="s">
         <v>57</v>
@@ -2107,7 +2116,7 @@
         <v>13</v>
       </c>
       <c r="J28" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
@@ -2124,22 +2133,22 @@
         <v>0.75</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G29" s="5" t="s">
         <v>17</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="I29" s="5" t="s">
         <v>13</v>
       </c>
       <c r="J29" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
@@ -2156,13 +2165,13 @@
         <v>0.7916666666678793</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H30" s="5" t="s">
         <v>12</v>
@@ -2171,7 +2180,7 @@
         <v>13</v>
       </c>
       <c r="J30" s="5" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
@@ -5075,10 +5084,10 @@
         <v>6</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>0</v>
@@ -5093,43 +5102,43 @@
         <v>3</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="T1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
@@ -5146,7 +5155,7 @@
         <v>11</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G2" s="5" t="b">
         <v>0</v>
@@ -5167,10 +5176,10 @@
         <v>12</v>
       </c>
       <c r="U2" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W2" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
@@ -5190,7 +5199,7 @@
         <v>17</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G3" s="5" t="b">
         <v>0</v>
@@ -5214,10 +5223,10 @@
         <v>12</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
@@ -5228,7 +5237,7 @@
         <v>13</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>25</v>
@@ -5237,7 +5246,7 @@
         <v>17</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G4" s="5" t="b">
         <v>0</v>
@@ -5261,10 +5270,10 @@
         <v>12</v>
       </c>
       <c r="U4" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W4" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
@@ -5284,7 +5293,7 @@
         <v>21</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G5" s="5" t="b">
         <v>0</v>
@@ -5308,13 +5317,13 @@
         <v>22</v>
       </c>
       <c r="U5" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="V5" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="W5" s="5" t="s">
         <v>116</v>
-      </c>
-      <c r="W5" s="5" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
@@ -5325,7 +5334,7 @@
         <v>13</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>38</v>
@@ -5334,7 +5343,7 @@
         <v>17</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G6" s="5" t="b">
         <v>0</v>
@@ -5355,30 +5364,30 @@
         <v>12</v>
       </c>
       <c r="U6" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W6" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G7" s="5" t="b">
         <v>0</v>
@@ -5402,11 +5411,11 @@
         <v>22</v>
       </c>
       <c r="U7" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="V7" s="11"/>
       <c r="W7" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
@@ -5426,7 +5435,7 @@
         <v>17</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G8" s="5" t="b">
         <v>0</v>
@@ -5450,30 +5459,30 @@
         <v>12</v>
       </c>
       <c r="U8" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W8" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="5" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G9" s="5" t="b">
         <v>0</v>
@@ -5494,13 +5503,13 @@
         <v>30.0</v>
       </c>
       <c r="T9" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="U9" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W9" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
@@ -5520,7 +5529,7 @@
         <v>17</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G10" s="5" t="b">
         <v>0</v>
@@ -5544,10 +5553,10 @@
         <v>12</v>
       </c>
       <c r="U10" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W10" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
@@ -5564,10 +5573,10 @@
         <v>66</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>71</v>
+        <v>126</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G11" s="5" t="b">
         <v>0</v>
@@ -5588,10 +5597,10 @@
         <v>57</v>
       </c>
       <c r="U11" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W11" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
@@ -5608,7 +5617,7 @@
         <v>69</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G12" s="5" t="b">
         <v>0</v>
@@ -5626,10 +5635,10 @@
         <v>0.6673611111109494</v>
       </c>
       <c r="U12" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W12" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
@@ -5643,13 +5652,13 @@
         <v>12</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>71</v>
+        <v>126</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G13" s="5" t="b">
         <v>0</v>
@@ -5673,15 +5682,15 @@
         <v>12</v>
       </c>
       <c r="U13" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W13" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>13</v>
@@ -5690,13 +5699,13 @@
         <v>12</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>71</v>
+        <v>126</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G14" s="5" t="b">
         <v>0</v>
@@ -5720,15 +5729,15 @@
         <v>12</v>
       </c>
       <c r="U14" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W14" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1">
       <c r="A15" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>13</v>
@@ -5737,13 +5746,13 @@
         <v>12</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G15" s="5" t="b">
         <v>0</v>
@@ -5767,30 +5776,30 @@
         <v>12</v>
       </c>
       <c r="U15" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W15" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G16" s="5" t="b">
         <v>0</v>
@@ -5814,15 +5823,15 @@
         <v>29</v>
       </c>
       <c r="U16" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W16" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>13</v>
@@ -5831,13 +5840,13 @@
         <v>68</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G17" s="5" t="b">
         <v>0</v>
@@ -5861,15 +5870,15 @@
         <v>12</v>
       </c>
       <c r="U17" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W17" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>13</v>
@@ -5878,13 +5887,13 @@
         <v>12</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>71</v>
+        <v>126</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G18" s="5" t="b">
         <v>0</v>
@@ -5908,15 +5917,15 @@
         <v>12</v>
       </c>
       <c r="U18" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W18" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>13</v>
@@ -5925,10 +5934,10 @@
         <v>68</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G19" s="5" t="b">
         <v>0</v>
@@ -5952,15 +5961,15 @@
         <v>12</v>
       </c>
       <c r="U19" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W19" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B20" s="5" t="s">
         <v>13</v>
@@ -5969,13 +5978,13 @@
         <v>12</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>71</v>
+        <v>126</v>
       </c>
       <c r="E20" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G20" s="5" t="b">
         <v>0</v>
@@ -5999,15 +6008,15 @@
         <v>12</v>
       </c>
       <c r="U20" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W20" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>13</v>
@@ -6016,13 +6025,13 @@
         <v>12</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>71</v>
+        <v>126</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G21" s="5" t="b">
         <v>0</v>
@@ -6046,30 +6055,30 @@
         <v>12</v>
       </c>
       <c r="U21" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W21" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G22" s="5" t="b">
         <v>0</v>
@@ -6090,30 +6099,30 @@
         <v>57</v>
       </c>
       <c r="U22" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W22" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="5" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G23" s="5" t="b">
         <v>0</v>
@@ -6134,10 +6143,10 @@
         <v>12</v>
       </c>
       <c r="U23" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W23" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
@@ -10917,22 +10926,22 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G1" s="5" t="b">
         <v>0</v>
@@ -10950,18 +10959,18 @@
         <v>0.7708333333321207</v>
       </c>
       <c r="T1" s="5" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="U1" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W1" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>13</v>
@@ -10970,13 +10979,13 @@
         <v>46</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G2" s="5" t="b">
         <v>0</v>
@@ -10997,30 +11006,30 @@
         <v>46</v>
       </c>
       <c r="U2" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W2" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G3" s="5" t="b">
         <v>0</v>
@@ -11041,30 +11050,30 @@
         <v>22</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G4" s="5" t="b">
         <v>0</v>
@@ -11083,18 +11092,18 @@
       </c>
       <c r="L4" s="2"/>
       <c r="T4" s="5" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="U4" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W4" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>13</v>
@@ -11103,13 +11112,13 @@
         <v>46</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G5" s="5" t="b">
         <v>0</v>
@@ -11130,13 +11139,13 @@
         <v>46</v>
       </c>
       <c r="U5" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W5" s="5"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>13</v>
@@ -11145,13 +11154,13 @@
         <v>12</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G6" s="5" t="b">
         <v>0</v>
@@ -11175,30 +11184,30 @@
         <v>12</v>
       </c>
       <c r="U6" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W6" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G7" s="5" t="b">
         <v>0</v>
@@ -11219,30 +11228,30 @@
         <v>22</v>
       </c>
       <c r="U7" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W7" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G8" s="5" t="b">
         <v>0</v>
@@ -11263,18 +11272,18 @@
         <v>60.0</v>
       </c>
       <c r="T8" s="5" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="U8" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W8" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>13</v>
@@ -11283,13 +11292,13 @@
         <v>12</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G9" s="5" t="b">
         <v>0</v>
@@ -11313,15 +11322,15 @@
         <v>12</v>
       </c>
       <c r="U9" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W9" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>13</v>
@@ -11330,13 +11339,13 @@
         <v>12</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G10" s="5" t="b">
         <v>0</v>
@@ -11360,15 +11369,15 @@
         <v>12</v>
       </c>
       <c r="U10" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W10" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>13</v>
@@ -11377,13 +11386,13 @@
         <v>12</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G11" s="5" t="b">
         <v>0</v>
@@ -11407,15 +11416,15 @@
         <v>12</v>
       </c>
       <c r="U11" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W11" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>13</v>
@@ -11424,13 +11433,13 @@
         <v>46</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G12" s="5" t="b">
         <v>0</v>
@@ -11451,15 +11460,15 @@
         <v>46</v>
       </c>
       <c r="U12" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W12" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>13</v>
@@ -11468,13 +11477,13 @@
         <v>12</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G13" s="5" t="b">
         <v>0</v>
@@ -11498,30 +11507,30 @@
         <v>12</v>
       </c>
       <c r="U13" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W13" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G14" s="5" t="b">
         <v>0</v>
@@ -11545,15 +11554,15 @@
         <v>12</v>
       </c>
       <c r="U14" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W14" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>13</v>
@@ -11562,10 +11571,10 @@
         <v>68</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G15" s="5" t="b">
         <v>0</v>
@@ -11583,15 +11592,15 @@
         <v>0.6673611111109494</v>
       </c>
       <c r="U15" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W15" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>13</v>
@@ -11600,10 +11609,10 @@
         <v>68</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G16" s="5" t="b">
         <v>0</v>
@@ -11621,15 +11630,15 @@
         <v>0.6673611111109494</v>
       </c>
       <c r="U16" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W16" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>13</v>
@@ -11638,13 +11647,13 @@
         <v>12</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G17" s="5" t="b">
         <v>0</v>
@@ -11668,15 +11677,15 @@
         <v>12</v>
       </c>
       <c r="U17" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W17" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>13</v>
@@ -11685,13 +11694,13 @@
         <v>46</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G18" s="5" t="b">
         <v>0</v>
@@ -11715,30 +11724,30 @@
         <v>46</v>
       </c>
       <c r="U18" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W18" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="E19" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G19" s="5" t="b">
         <v>0</v>
@@ -11759,18 +11768,18 @@
         <v>30.0</v>
       </c>
       <c r="T19" s="5" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="U19" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W19" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B20" s="5" t="s">
         <v>13</v>
@@ -11779,10 +11788,10 @@
         <v>68</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G20" s="5" t="b">
         <v>0</v>
@@ -11800,15 +11809,15 @@
         <v>0.6673611111109494</v>
       </c>
       <c r="U20" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W20" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>13</v>
@@ -11823,7 +11832,7 @@
         <v>17</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G21" s="5" t="b">
         <v>0</v>
@@ -11847,15 +11856,15 @@
         <v>12</v>
       </c>
       <c r="U21" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W21" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>13</v>
@@ -11870,7 +11879,7 @@
         <v>17</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G22" s="5" t="b">
         <v>0</v>
@@ -11894,30 +11903,30 @@
         <v>12</v>
       </c>
       <c r="U22" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W22" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="5" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="E23" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G23" s="5" t="b">
         <v>0</v>
@@ -11941,30 +11950,30 @@
         <v>12</v>
       </c>
       <c r="U23" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W23" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="5" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="E24" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G24" s="5" t="b">
         <v>0</v>
@@ -11988,30 +11997,30 @@
         <v>12</v>
       </c>
       <c r="U24" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W24" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="5" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="E25" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G25" s="5" t="b">
         <v>0</v>
@@ -12035,30 +12044,30 @@
         <v>12</v>
       </c>
       <c r="U25" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W25" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="5" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G26" s="5" t="b">
         <v>0</v>
@@ -12076,21 +12085,21 @@
         <v>0.6875</v>
       </c>
       <c r="T26" s="5" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="U26" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="V26" s="12" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="W26" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="5" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>13</v>
@@ -12099,13 +12108,13 @@
         <v>46</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="E27" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G27" s="5" t="b">
         <v>0</v>
@@ -12126,28 +12135,28 @@
         <v>46</v>
       </c>
       <c r="U27" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W27" s="5"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="5" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="E28" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G28" s="5" t="b">
         <v>0</v>
@@ -12165,30 +12174,30 @@
         <v>0.6736111111094942</v>
       </c>
       <c r="U28" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W28" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="5" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="E29" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G29" s="5" t="b">
         <v>0</v>
@@ -12206,33 +12215,33 @@
         <v>0.8125</v>
       </c>
       <c r="T29" s="5" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="U29" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W29" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="5" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G30" s="5" t="b">
         <v>0</v>
@@ -12256,30 +12265,30 @@
         <v>12</v>
       </c>
       <c r="U30" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W30" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="5" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="E31" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G31" s="5" t="b">
         <v>0</v>
@@ -12303,21 +12312,21 @@
         <v>22</v>
       </c>
       <c r="U31" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W31" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="5" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>16</v>
@@ -12326,7 +12335,7 @@
         <v>17</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G32" s="5" t="b">
         <v>0</v>
@@ -12350,30 +12359,30 @@
         <v>12</v>
       </c>
       <c r="U32" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W32" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="5" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G33" s="5" t="b">
         <v>0</v>
@@ -12391,24 +12400,24 @@
         <v>0.3958333333321207</v>
       </c>
       <c r="T33" s="5" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="U33" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W33" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="5" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>16</v>
@@ -12417,7 +12426,7 @@
         <v>17</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G34" s="5" t="b">
         <v>0</v>
@@ -12441,30 +12450,30 @@
         <v>12</v>
       </c>
       <c r="U34" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W34" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="5" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="B35" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="E35" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G35" s="5" t="b">
         <v>0</v>
@@ -12485,24 +12494,24 @@
         <v>30.0</v>
       </c>
       <c r="T35" s="5" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="U35" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W35" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="5" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="B36" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>16</v>
@@ -12511,7 +12520,7 @@
         <v>17</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G36" s="5" t="b">
         <v>0</v>
@@ -12535,15 +12544,15 @@
         <v>12</v>
       </c>
       <c r="U36" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W36" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="5" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B37" s="5" t="s">
         <v>13</v>
@@ -12552,13 +12561,13 @@
         <v>46</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="E37" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G37" s="5" t="b">
         <v>0</v>
@@ -12579,25 +12588,25 @@
         <v>46</v>
       </c>
       <c r="U37" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W37" s="5"/>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="5" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="B38" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="F38" s="5"/>
       <c r="G38" s="5" t="b">
@@ -12619,21 +12628,21 @@
         <v>22</v>
       </c>
       <c r="U38" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W38" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="5" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>16</v>
@@ -12642,7 +12651,7 @@
         <v>17</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G39" s="5" t="b">
         <v>0</v>
@@ -12666,30 +12675,30 @@
         <v>12</v>
       </c>
       <c r="U39" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W39" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="5" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="B40" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="E40" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G40" s="5" t="b">
         <v>0</v>
@@ -12713,27 +12722,27 @@
         <v>12</v>
       </c>
       <c r="U40" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W40" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="5" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="B41" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G41" s="5" t="b">
         <v>0</v>
@@ -12754,10 +12763,10 @@
         <v>12</v>
       </c>
       <c r="U41" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W41" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="42">
@@ -12774,13 +12783,13 @@
         <v>0.625</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="H42" s="5" t="s">
         <v>22</v>
@@ -12789,7 +12798,7 @@
         <v>13</v>
       </c>
       <c r="J42" s="5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -12823,227 +12832,227 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="M1" s="13" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="M2" s="14" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
     <row r="5">
       <c r="M5" s="15" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="M20" s="5" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="8" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="8" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="8" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="8" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="8" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="8" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="8" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1"/>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="8" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="8" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="8" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="8" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="8" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="8" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="8" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1"/>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="8" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="8" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="8" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="8" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1"/>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="8" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="8" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="8" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="8" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="8" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="8" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
Bugle June 7, 2026
</commit_message>
<xml_diff>
--- a/Troop 79 Bugle Calendar for ICS Feed.xlsx
+++ b/Troop 79 Bugle Calendar for ICS Feed.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="810" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="816" uniqueCount="278">
   <si>
     <t>start_date</t>
   </si>
@@ -237,166 +237,184 @@
     <t>bc71eaf15abdc3a5673e8d6721de7f00@sheet2ics</t>
   </si>
   <si>
+    <t>Pack 179 Cross Over</t>
+  </si>
+  <si>
+    <t>AOL Crossover Cermony will be at about 1:15</t>
+  </si>
+  <si>
+    <t>Grant Park Picnic Area 6, 215 S Lake Dr.</t>
+  </si>
+  <si>
+    <t>Ceremony</t>
+  </si>
+  <si>
+    <t>cd0d9bd15cec2308a9b45c5e3eff05ef@sheet2ics</t>
+  </si>
+  <si>
     <t>Woodwork MB - Makeup / Finishup</t>
   </si>
   <si>
     <t>849dd533a5088b786aa5d3d25ee9b681@sheet2ics</t>
   </si>
   <si>
+    <t>Camp Physicals / HAT Prep / Open Advancement</t>
+  </si>
+  <si>
+    <t>7222db9d6348d0631faa2378d1c8ee88@sheet2ics</t>
+  </si>
+  <si>
+    <t>High Adventure Trip</t>
+  </si>
+  <si>
+    <t>05ea088280e099fce97694e4f6ddf12f@sheet2ics</t>
+  </si>
+  <si>
+    <t>BWCA</t>
+  </si>
+  <si>
+    <t>02e52d7fe6a30e4623930f66937f1701@sheet2ics</t>
+  </si>
+  <si>
+    <t>Camp Physicals / Open Advancement</t>
+  </si>
+  <si>
+    <t>107491addb3b9576ed2b5be31a06f102@sheet2ics</t>
+  </si>
+  <si>
+    <t>Fourth of July</t>
+  </si>
+  <si>
+    <t>290ab3dfb24f23c44b85ee236bcbf1ee@sheet2ics</t>
+  </si>
+  <si>
+    <t>Prep for Summer Camp</t>
+  </si>
+  <si>
+    <t>38b737926b25d932e994b62a7b15a29d@sheet2ics</t>
+  </si>
+  <si>
+    <t>0df89d505ff7db5d0fd6917fadcafbeb@sheet2ics</t>
+  </si>
+  <si>
+    <t>Summer Camp - Tesomas</t>
+  </si>
+  <si>
+    <t>Tesomas Scout Reservation</t>
+  </si>
+  <si>
+    <t>5403 Spider Lake Rd, Rhinelander, WI 54501</t>
+  </si>
+  <si>
+    <t>1b0cff4a338d00c5b8e27f8b9a02eac4@sheet2ics</t>
+  </si>
+  <si>
+    <t>Rummage Sale</t>
+  </si>
+  <si>
+    <t>All Day Rummage Sale</t>
+  </si>
+  <si>
+    <t>Fund Raiser</t>
+  </si>
+  <si>
+    <t>2a356e920aad675a7efea5fc90141738@sheet2ics</t>
+  </si>
+  <si>
+    <t>Court of Honor</t>
+  </si>
+  <si>
+    <t>Grant Park Picnic Area</t>
+  </si>
+  <si>
+    <t>Grant Park Picnic Area with Shelter</t>
+  </si>
+  <si>
+    <t>11a5cb096a7f6578a8ef2d5ed2b76687@sheet2ics</t>
+  </si>
+  <si>
+    <t>timezone</t>
+  </si>
+  <si>
+    <t>all_day</t>
+  </si>
+  <si>
+    <t>due_date</t>
+  </si>
+  <si>
+    <t>due_time</t>
+  </si>
+  <si>
+    <t>recurrence_rule</t>
+  </si>
+  <si>
+    <t>recurrence_until</t>
+  </si>
+  <si>
+    <t>recurrence_count</t>
+  </si>
+  <si>
+    <t>exdates</t>
+  </si>
+  <si>
+    <t>alarm_minutes_before</t>
+  </si>
+  <si>
+    <t>attendees</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>url</t>
+  </si>
+  <si>
+    <t>organizer_email</t>
+  </si>
+  <si>
+    <t>notes_internal</t>
+  </si>
+  <si>
+    <t>America/Chicago</t>
+  </si>
+  <si>
+    <t>CONFIRMED</t>
+  </si>
+  <si>
+    <t>bsatroop79bg@gmail.com</t>
+  </si>
+  <si>
+    <t>Troop Meeting - Wood Working MB</t>
+  </si>
+  <si>
+    <t>https://band.us/band/93239709/schedule/4%2F93239709%2F961498689%2F19700101</t>
+  </si>
+  <si>
+    <t>8f47e9ac8233a825ca1e54ece63c20ca@sheet2ics</t>
+  </si>
+  <si>
+    <t>Service Project - Oakleaf Trail Cleanup</t>
+  </si>
+  <si>
+    <t>Oakleaf Trail Cleanup</t>
+  </si>
+  <si>
+    <t>Colectivo Lakefront</t>
+  </si>
+  <si>
+    <t>b488cfbac2b9a8a809c579b888ed61ee@sheet2ics</t>
+  </si>
+  <si>
+    <t>Pancake Breakfast Fund Raiser</t>
+  </si>
+  <si>
+    <t>Annual Pancake Breakfast</t>
+  </si>
+  <si>
+    <t>TBD</t>
+  </si>
+  <si>
     <t>Prepare for High Adventure Trip</t>
-  </si>
-  <si>
-    <t>7222db9d6348d0631faa2378d1c8ee88@sheet2ics</t>
-  </si>
-  <si>
-    <t>High Adventure Trip</t>
-  </si>
-  <si>
-    <t>BWCA</t>
-  </si>
-  <si>
-    <t>02e52d7fe6a30e4623930f66937f1701@sheet2ics</t>
-  </si>
-  <si>
-    <t>05ea088280e099fce97694e4f6ddf12f@sheet2ics</t>
-  </si>
-  <si>
-    <t>Camp Physicals</t>
-  </si>
-  <si>
-    <t>107491addb3b9576ed2b5be31a06f102@sheet2ics</t>
-  </si>
-  <si>
-    <t>Fourth of July</t>
-  </si>
-  <si>
-    <t>290ab3dfb24f23c44b85ee236bcbf1ee@sheet2ics</t>
-  </si>
-  <si>
-    <t>Prep for Summer Camp</t>
-  </si>
-  <si>
-    <t>38b737926b25d932e994b62a7b15a29d@sheet2ics</t>
-  </si>
-  <si>
-    <t>0df89d505ff7db5d0fd6917fadcafbeb@sheet2ics</t>
-  </si>
-  <si>
-    <t>Summer Camp - Tesomas</t>
-  </si>
-  <si>
-    <t>Tesomas Scout Reservation</t>
-  </si>
-  <si>
-    <t>5403 Spider Lake Rd, Rhinelander, WI 54501</t>
-  </si>
-  <si>
-    <t>1b0cff4a338d00c5b8e27f8b9a02eac4@sheet2ics</t>
-  </si>
-  <si>
-    <t>Rummage Sale</t>
-  </si>
-  <si>
-    <t>All Day Rummage Sale</t>
-  </si>
-  <si>
-    <t>Fund Raiser</t>
-  </si>
-  <si>
-    <t>2a356e920aad675a7efea5fc90141738@sheet2ics</t>
-  </si>
-  <si>
-    <t>Court of Honor</t>
-  </si>
-  <si>
-    <t>Grant Park Picnic Area</t>
-  </si>
-  <si>
-    <t>Grant Park Picnic Area with Shelter</t>
-  </si>
-  <si>
-    <t>11a5cb096a7f6578a8ef2d5ed2b76687@sheet2ics</t>
-  </si>
-  <si>
-    <t>timezone</t>
-  </si>
-  <si>
-    <t>all_day</t>
-  </si>
-  <si>
-    <t>due_date</t>
-  </si>
-  <si>
-    <t>due_time</t>
-  </si>
-  <si>
-    <t>recurrence_rule</t>
-  </si>
-  <si>
-    <t>recurrence_until</t>
-  </si>
-  <si>
-    <t>recurrence_count</t>
-  </si>
-  <si>
-    <t>exdates</t>
-  </si>
-  <si>
-    <t>alarm_minutes_before</t>
-  </si>
-  <si>
-    <t>attendees</t>
-  </si>
-  <si>
-    <t>status</t>
-  </si>
-  <si>
-    <t>url</t>
-  </si>
-  <si>
-    <t>organizer_email</t>
-  </si>
-  <si>
-    <t>notes_internal</t>
-  </si>
-  <si>
-    <t>America/Chicago</t>
-  </si>
-  <si>
-    <t>CONFIRMED</t>
-  </si>
-  <si>
-    <t>bsatroop79bg@gmail.com</t>
-  </si>
-  <si>
-    <t>Troop Meeting - Wood Working MB</t>
-  </si>
-  <si>
-    <t>https://band.us/band/93239709/schedule/4%2F93239709%2F961498689%2F19700101</t>
-  </si>
-  <si>
-    <t>8f47e9ac8233a825ca1e54ece63c20ca@sheet2ics</t>
-  </si>
-  <si>
-    <t>Service Project - Oakleaf Trail Cleanup</t>
-  </si>
-  <si>
-    <t>Oakleaf Trail Cleanup</t>
-  </si>
-  <si>
-    <t>Colectivo Lakefront</t>
-  </si>
-  <si>
-    <t>b488cfbac2b9a8a809c579b888ed61ee@sheet2ics</t>
-  </si>
-  <si>
-    <t>Pancake Breakfast Fund Raiser</t>
-  </si>
-  <si>
-    <t>Annual Pancake Breakfast</t>
-  </si>
-  <si>
-    <t>TBD</t>
   </si>
   <si>
     <t>8ab1c36a61c104dc8f881142028eb1b5@sheet2ics</t>
@@ -1836,45 +1854,45 @@
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="2">
-        <v>46180.0</v>
+        <v>46179.0</v>
       </c>
       <c r="B20" s="3">
-        <v>0.6666666666678793</v>
+        <v>0.4583333333321207</v>
       </c>
       <c r="C20" s="2">
-        <v>46180.0</v>
-      </c>
-      <c r="D20" s="4">
-        <v>0.7291666666678793</v>
+        <v>46179.0</v>
+      </c>
+      <c r="D20" s="3">
+        <v>0.5833333333321207</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>12</v>
+        <v>73</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>17</v>
+        <v>75</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>12</v>
+        <v>76</v>
       </c>
       <c r="I20" s="5" t="s">
         <v>13</v>
       </c>
       <c r="J20" s="5" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="2">
-        <v>46187.0</v>
+        <v>46180.0</v>
       </c>
       <c r="B21" s="3">
         <v>0.6666666666678793</v>
       </c>
       <c r="C21" s="2">
-        <v>46187.0</v>
+        <v>46180.0</v>
       </c>
       <c r="D21" s="4">
         <v>0.7291666666678793</v>
@@ -1883,7 +1901,7 @@
         <v>12</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="G21" s="5" t="s">
         <v>17</v>
@@ -1895,39 +1913,39 @@
         <v>13</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="2">
-        <v>46193.0</v>
+        <v>46187.0</v>
       </c>
       <c r="B22" s="3">
-        <v>0.2916666666678793</v>
+        <v>0.6666666666678793</v>
       </c>
       <c r="C22" s="2">
-        <v>46200.0</v>
+        <v>46187.0</v>
       </c>
       <c r="D22" s="4">
-        <v>0.625</v>
+        <v>0.7291666666678793</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>77</v>
+        <v>12</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>78</v>
+        <v>17</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="I22" s="5" t="s">
         <v>13</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
@@ -1947,7 +1965,7 @@
         <v>68</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="G23" s="5" t="s">
         <v>17</v>
@@ -1959,59 +1977,62 @@
         <v>13</v>
       </c>
       <c r="J23" s="5" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="2">
-        <v>46201.0</v>
+        <v>46193.0</v>
       </c>
       <c r="B24" s="3">
-        <v>0.6666666666678793</v>
+        <v>0.2916666666678793</v>
       </c>
       <c r="C24" s="2">
-        <v>46201.0</v>
+        <v>46200.0</v>
       </c>
       <c r="D24" s="4">
-        <v>0.7291666666678793</v>
+        <v>0.625</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>12</v>
+        <v>82</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>17</v>
+        <v>84</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="I24" s="5" t="s">
         <v>13</v>
       </c>
       <c r="J24" s="5" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="2">
-        <v>46208.0</v>
+        <v>46201.0</v>
       </c>
       <c r="B25" s="3">
         <v>0.6666666666678793</v>
       </c>
       <c r="C25" s="2">
-        <v>46208.0</v>
+        <v>46201.0</v>
       </c>
       <c r="D25" s="4">
-        <v>0.6770833333321207</v>
+        <v>0.7291666666678793</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>68</v>
+        <v>12</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>83</v>
+        <v>86</v>
+      </c>
+      <c r="G25" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="H25" s="5" t="s">
         <v>12</v>
@@ -2020,30 +2041,27 @@
         <v>13</v>
       </c>
       <c r="J25" s="5" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="2">
-        <v>46215.0</v>
+        <v>46208.0</v>
       </c>
       <c r="B26" s="3">
         <v>0.6666666666678793</v>
       </c>
       <c r="C26" s="2">
-        <v>46215.0</v>
+        <v>46208.0</v>
       </c>
       <c r="D26" s="4">
-        <v>0.7291666666678793</v>
+        <v>0.6770833333321207</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>12</v>
+        <v>68</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="G26" s="5" t="s">
-        <v>17</v>
+        <v>88</v>
       </c>
       <c r="H26" s="5" t="s">
         <v>12</v>
@@ -2052,18 +2070,18 @@
         <v>13</v>
       </c>
       <c r="J26" s="5" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="2">
-        <v>46222.0</v>
+        <v>46215.0</v>
       </c>
       <c r="B27" s="3">
         <v>0.6666666666678793</v>
       </c>
       <c r="C27" s="2">
-        <v>46222.0</v>
+        <v>46215.0</v>
       </c>
       <c r="D27" s="4">
         <v>0.7291666666678793</v>
@@ -2072,7 +2090,7 @@
         <v>12</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="G27" s="5" t="s">
         <v>17</v>
@@ -2084,107 +2102,136 @@
         <v>13</v>
       </c>
       <c r="J27" s="5" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="2">
-        <v>46229.0</v>
+        <v>46222.0</v>
       </c>
       <c r="B28" s="3">
-        <v>0.2916666666678793</v>
+        <v>0.6666666666678793</v>
       </c>
       <c r="C28" s="2">
-        <v>46235.0</v>
-      </c>
-      <c r="D28" s="3">
-        <v>0.5416666666678793</v>
+        <v>46222.0</v>
+      </c>
+      <c r="D28" s="4">
+        <v>0.7291666666678793</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>88</v>
+        <v>12</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>90</v>
+        <v>17</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>57</v>
+        <v>12</v>
       </c>
       <c r="I28" s="5" t="s">
         <v>13</v>
       </c>
       <c r="J28" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="2">
-        <v>46263.0</v>
+        <v>46229.0</v>
       </c>
       <c r="B29" s="3">
-        <v>0.375</v>
+        <v>0.2916666666678793</v>
       </c>
       <c r="C29" s="2">
-        <v>46263.0</v>
-      </c>
-      <c r="D29" s="4">
-        <v>0.75</v>
+        <v>46235.0</v>
+      </c>
+      <c r="D29" s="3">
+        <v>0.5416666666678793</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>17</v>
+        <v>95</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>94</v>
+        <v>57</v>
       </c>
       <c r="I29" s="5" t="s">
         <v>13</v>
       </c>
       <c r="J29" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="7">
-        <v>46278.0</v>
-      </c>
-      <c r="B30" s="4">
-        <v>0.625</v>
-      </c>
-      <c r="C30" s="7">
-        <v>46278.0</v>
-      </c>
-      <c r="D30" s="3">
-        <v>0.7916666666678793</v>
+      <c r="A30" s="2">
+        <v>46263.0</v>
+      </c>
+      <c r="B30" s="3">
+        <v>0.375</v>
+      </c>
+      <c r="C30" s="2">
+        <v>46263.0</v>
+      </c>
+      <c r="D30" s="4">
+        <v>0.75</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>98</v>
+        <v>17</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>12</v>
+        <v>99</v>
       </c>
       <c r="I30" s="5" t="s">
         <v>13</v>
       </c>
       <c r="J30" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="I31" s="8"/>
+      <c r="A31" s="7">
+        <v>46278.0</v>
+      </c>
+      <c r="B31" s="4">
+        <v>0.625</v>
+      </c>
+      <c r="C31" s="7">
+        <v>46278.0</v>
+      </c>
+      <c r="D31" s="3">
+        <v>0.7916666666678793</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="G31" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="H31" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I31" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="J31" s="5" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="I32" s="8"/>
@@ -5023,11 +5070,14 @@
     </row>
     <row r="977" ht="15.75" customHeight="1">
       <c r="I977" s="8"/>
+    </row>
+    <row r="978" ht="15.75" customHeight="1">
+      <c r="I978" s="8"/>
     </row>
   </sheetData>
   <autoFilter ref="$E$1:$H$1"/>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I2:I977">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I2:I978">
       <formula1>"VEVENT,VTODO"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5084,10 +5134,10 @@
         <v>6</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>0</v>
@@ -5102,43 +5152,43 @@
         <v>3</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="T1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
@@ -5155,7 +5205,7 @@
         <v>11</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G2" s="5" t="b">
         <v>0</v>
@@ -5176,10 +5226,10 @@
         <v>12</v>
       </c>
       <c r="U2" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W2" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
@@ -5199,7 +5249,7 @@
         <v>17</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G3" s="5" t="b">
         <v>0</v>
@@ -5223,10 +5273,10 @@
         <v>12</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
@@ -5237,7 +5287,7 @@
         <v>13</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>25</v>
@@ -5246,7 +5296,7 @@
         <v>17</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G4" s="5" t="b">
         <v>0</v>
@@ -5270,10 +5320,10 @@
         <v>12</v>
       </c>
       <c r="U4" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W4" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
@@ -5293,7 +5343,7 @@
         <v>21</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G5" s="5" t="b">
         <v>0</v>
@@ -5317,13 +5367,13 @@
         <v>22</v>
       </c>
       <c r="U5" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="V5" s="10" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="W5" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
@@ -5334,7 +5384,7 @@
         <v>13</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>38</v>
@@ -5343,7 +5393,7 @@
         <v>17</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G6" s="5" t="b">
         <v>0</v>
@@ -5364,30 +5414,30 @@
         <v>12</v>
       </c>
       <c r="U6" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W6" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="5" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G7" s="5" t="b">
         <v>0</v>
@@ -5411,11 +5461,11 @@
         <v>22</v>
       </c>
       <c r="U7" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="V7" s="11"/>
       <c r="W7" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
@@ -5435,7 +5485,7 @@
         <v>17</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G8" s="5" t="b">
         <v>0</v>
@@ -5459,30 +5509,30 @@
         <v>12</v>
       </c>
       <c r="U8" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W8" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="5" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G9" s="5" t="b">
         <v>0</v>
@@ -5503,13 +5553,13 @@
         <v>30.0</v>
       </c>
       <c r="T9" s="5" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="U9" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W9" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
@@ -5529,7 +5579,7 @@
         <v>17</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G10" s="5" t="b">
         <v>0</v>
@@ -5553,10 +5603,10 @@
         <v>12</v>
       </c>
       <c r="U10" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W10" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
@@ -5573,10 +5623,10 @@
         <v>66</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G11" s="5" t="b">
         <v>0</v>
@@ -5597,10 +5647,10 @@
         <v>57</v>
       </c>
       <c r="U11" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W11" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
@@ -5617,7 +5667,7 @@
         <v>69</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G12" s="5" t="b">
         <v>0</v>
@@ -5635,10 +5685,10 @@
         <v>0.6673611111109494</v>
       </c>
       <c r="U12" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W12" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
@@ -5652,13 +5702,13 @@
         <v>12</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G13" s="5" t="b">
         <v>0</v>
@@ -5682,15 +5732,15 @@
         <v>12</v>
       </c>
       <c r="U13" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W13" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="5" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>13</v>
@@ -5699,13 +5749,13 @@
         <v>12</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G14" s="5" t="b">
         <v>0</v>
@@ -5729,15 +5779,15 @@
         <v>12</v>
       </c>
       <c r="U14" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W14" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1">
       <c r="A15" s="5" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>13</v>
@@ -5746,13 +5796,13 @@
         <v>12</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>75</v>
+        <v>132</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G15" s="5" t="b">
         <v>0</v>
@@ -5776,30 +5826,30 @@
         <v>12</v>
       </c>
       <c r="U15" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W15" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="5" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G16" s="5" t="b">
         <v>0</v>
@@ -5823,15 +5873,15 @@
         <v>29</v>
       </c>
       <c r="U16" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W16" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="5" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>13</v>
@@ -5840,13 +5890,13 @@
         <v>68</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G17" s="5" t="b">
         <v>0</v>
@@ -5870,15 +5920,15 @@
         <v>12</v>
       </c>
       <c r="U17" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W17" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="5" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>13</v>
@@ -5887,13 +5937,13 @@
         <v>12</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G18" s="5" t="b">
         <v>0</v>
@@ -5917,15 +5967,15 @@
         <v>12</v>
       </c>
       <c r="U18" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W18" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="5" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>13</v>
@@ -5934,10 +5984,10 @@
         <v>68</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G19" s="5" t="b">
         <v>0</v>
@@ -5961,15 +6011,15 @@
         <v>12</v>
       </c>
       <c r="U19" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W19" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="5" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B20" s="5" t="s">
         <v>13</v>
@@ -5978,13 +6028,13 @@
         <v>12</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="E20" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G20" s="5" t="b">
         <v>0</v>
@@ -6008,15 +6058,15 @@
         <v>12</v>
       </c>
       <c r="U20" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W20" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="5" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>13</v>
@@ -6025,13 +6075,13 @@
         <v>12</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G21" s="5" t="b">
         <v>0</v>
@@ -6055,30 +6105,30 @@
         <v>12</v>
       </c>
       <c r="U21" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W21" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="5" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G22" s="5" t="b">
         <v>0</v>
@@ -6099,30 +6149,30 @@
         <v>57</v>
       </c>
       <c r="U22" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W22" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="5" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G23" s="5" t="b">
         <v>0</v>
@@ -6143,10 +6193,10 @@
         <v>12</v>
       </c>
       <c r="U23" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W23" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
@@ -10926,22 +10976,22 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G1" s="5" t="b">
         <v>0</v>
@@ -10959,18 +11009,18 @@
         <v>0.7708333333321207</v>
       </c>
       <c r="T1" s="5" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="U1" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W1" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>13</v>
@@ -10979,13 +11029,13 @@
         <v>46</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G2" s="5" t="b">
         <v>0</v>
@@ -11006,30 +11056,30 @@
         <v>46</v>
       </c>
       <c r="U2" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W2" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G3" s="5" t="b">
         <v>0</v>
@@ -11050,30 +11100,30 @@
         <v>22</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G4" s="5" t="b">
         <v>0</v>
@@ -11092,18 +11142,18 @@
       </c>
       <c r="L4" s="2"/>
       <c r="T4" s="5" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="U4" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W4" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>13</v>
@@ -11112,13 +11162,13 @@
         <v>46</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G5" s="5" t="b">
         <v>0</v>
@@ -11139,13 +11189,13 @@
         <v>46</v>
       </c>
       <c r="U5" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W5" s="5"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>13</v>
@@ -11154,13 +11204,13 @@
         <v>12</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G6" s="5" t="b">
         <v>0</v>
@@ -11184,30 +11234,30 @@
         <v>12</v>
       </c>
       <c r="U6" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W6" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G7" s="5" t="b">
         <v>0</v>
@@ -11228,30 +11278,30 @@
         <v>22</v>
       </c>
       <c r="U7" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W7" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G8" s="5" t="b">
         <v>0</v>
@@ -11272,18 +11322,18 @@
         <v>60.0</v>
       </c>
       <c r="T8" s="5" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="U8" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W8" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>13</v>
@@ -11292,13 +11342,13 @@
         <v>12</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G9" s="5" t="b">
         <v>0</v>
@@ -11322,15 +11372,15 @@
         <v>12</v>
       </c>
       <c r="U9" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W9" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>13</v>
@@ -11339,13 +11389,13 @@
         <v>12</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G10" s="5" t="b">
         <v>0</v>
@@ -11369,15 +11419,15 @@
         <v>12</v>
       </c>
       <c r="U10" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W10" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>13</v>
@@ -11386,13 +11436,13 @@
         <v>12</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G11" s="5" t="b">
         <v>0</v>
@@ -11416,15 +11466,15 @@
         <v>12</v>
       </c>
       <c r="U11" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W11" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>13</v>
@@ -11433,13 +11483,13 @@
         <v>46</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G12" s="5" t="b">
         <v>0</v>
@@ -11460,15 +11510,15 @@
         <v>46</v>
       </c>
       <c r="U12" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W12" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>13</v>
@@ -11477,13 +11527,13 @@
         <v>12</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G13" s="5" t="b">
         <v>0</v>
@@ -11507,30 +11557,30 @@
         <v>12</v>
       </c>
       <c r="U13" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W13" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G14" s="5" t="b">
         <v>0</v>
@@ -11554,15 +11604,15 @@
         <v>12</v>
       </c>
       <c r="U14" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W14" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>13</v>
@@ -11571,10 +11621,10 @@
         <v>68</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G15" s="5" t="b">
         <v>0</v>
@@ -11592,15 +11642,15 @@
         <v>0.6673611111109494</v>
       </c>
       <c r="U15" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W15" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>13</v>
@@ -11609,10 +11659,10 @@
         <v>68</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G16" s="5" t="b">
         <v>0</v>
@@ -11630,15 +11680,15 @@
         <v>0.6673611111109494</v>
       </c>
       <c r="U16" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W16" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>13</v>
@@ -11647,13 +11697,13 @@
         <v>12</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G17" s="5" t="b">
         <v>0</v>
@@ -11677,15 +11727,15 @@
         <v>12</v>
       </c>
       <c r="U17" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W17" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>13</v>
@@ -11694,13 +11744,13 @@
         <v>46</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G18" s="5" t="b">
         <v>0</v>
@@ -11724,30 +11774,30 @@
         <v>46</v>
       </c>
       <c r="U18" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W18" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="E19" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G19" s="5" t="b">
         <v>0</v>
@@ -11768,18 +11818,18 @@
         <v>30.0</v>
       </c>
       <c r="T19" s="5" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="U19" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W19" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="B20" s="5" t="s">
         <v>13</v>
@@ -11788,10 +11838,10 @@
         <v>68</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G20" s="5" t="b">
         <v>0</v>
@@ -11809,15 +11859,15 @@
         <v>0.6673611111109494</v>
       </c>
       <c r="U20" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W20" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>13</v>
@@ -11832,7 +11882,7 @@
         <v>17</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G21" s="5" t="b">
         <v>0</v>
@@ -11856,15 +11906,15 @@
         <v>12</v>
       </c>
       <c r="U21" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W21" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>13</v>
@@ -11879,7 +11929,7 @@
         <v>17</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G22" s="5" t="b">
         <v>0</v>
@@ -11903,30 +11953,30 @@
         <v>12</v>
       </c>
       <c r="U22" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W22" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="5" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="E23" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G23" s="5" t="b">
         <v>0</v>
@@ -11950,30 +12000,30 @@
         <v>12</v>
       </c>
       <c r="U23" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W23" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="5" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="E24" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G24" s="5" t="b">
         <v>0</v>
@@ -11997,30 +12047,30 @@
         <v>12</v>
       </c>
       <c r="U24" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W24" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="5" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="E25" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G25" s="5" t="b">
         <v>0</v>
@@ -12044,30 +12094,30 @@
         <v>12</v>
       </c>
       <c r="U25" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W25" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="5" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G26" s="5" t="b">
         <v>0</v>
@@ -12085,21 +12135,21 @@
         <v>0.6875</v>
       </c>
       <c r="T26" s="5" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="U26" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="V26" s="12" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="W26" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="5" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>13</v>
@@ -12108,13 +12158,13 @@
         <v>46</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="E27" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G27" s="5" t="b">
         <v>0</v>
@@ -12135,28 +12185,28 @@
         <v>46</v>
       </c>
       <c r="U27" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W27" s="5"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="5" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="E28" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G28" s="5" t="b">
         <v>0</v>
@@ -12174,30 +12224,30 @@
         <v>0.6736111111094942</v>
       </c>
       <c r="U28" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W28" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="5" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="E29" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G29" s="5" t="b">
         <v>0</v>
@@ -12215,33 +12265,33 @@
         <v>0.8125</v>
       </c>
       <c r="T29" s="5" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="U29" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W29" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="5" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G30" s="5" t="b">
         <v>0</v>
@@ -12265,30 +12315,30 @@
         <v>12</v>
       </c>
       <c r="U30" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W30" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="5" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="E31" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G31" s="5" t="b">
         <v>0</v>
@@ -12312,21 +12362,21 @@
         <v>22</v>
       </c>
       <c r="U31" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W31" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="5" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>16</v>
@@ -12335,7 +12385,7 @@
         <v>17</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G32" s="5" t="b">
         <v>0</v>
@@ -12359,30 +12409,30 @@
         <v>12</v>
       </c>
       <c r="U32" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W32" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="5" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G33" s="5" t="b">
         <v>0</v>
@@ -12400,24 +12450,24 @@
         <v>0.3958333333321207</v>
       </c>
       <c r="T33" s="5" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="U33" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W33" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="5" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>16</v>
@@ -12426,7 +12476,7 @@
         <v>17</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G34" s="5" t="b">
         <v>0</v>
@@ -12450,30 +12500,30 @@
         <v>12</v>
       </c>
       <c r="U34" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W34" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="5" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="B35" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="E35" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G35" s="5" t="b">
         <v>0</v>
@@ -12494,24 +12544,24 @@
         <v>30.0</v>
       </c>
       <c r="T35" s="5" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="U35" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W35" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="5" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="B36" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>16</v>
@@ -12520,7 +12570,7 @@
         <v>17</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G36" s="5" t="b">
         <v>0</v>
@@ -12544,15 +12594,15 @@
         <v>12</v>
       </c>
       <c r="U36" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W36" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="5" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="B37" s="5" t="s">
         <v>13</v>
@@ -12561,13 +12611,13 @@
         <v>46</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="E37" s="5" t="s">
         <v>21</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G37" s="5" t="b">
         <v>0</v>
@@ -12588,25 +12638,25 @@
         <v>46</v>
       </c>
       <c r="U37" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W37" s="5"/>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="5" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="B38" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="F38" s="5"/>
       <c r="G38" s="5" t="b">
@@ -12628,21 +12678,21 @@
         <v>22</v>
       </c>
       <c r="U38" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W38" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="5" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>16</v>
@@ -12651,7 +12701,7 @@
         <v>17</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G39" s="5" t="b">
         <v>0</v>
@@ -12675,30 +12725,30 @@
         <v>12</v>
       </c>
       <c r="U39" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W39" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="5" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="B40" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="E40" s="5" t="s">
         <v>17</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G40" s="5" t="b">
         <v>0</v>
@@ -12722,27 +12772,27 @@
         <v>12</v>
       </c>
       <c r="U40" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W40" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="5" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="B41" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="G41" s="5" t="b">
         <v>0</v>
@@ -12763,10 +12813,10 @@
         <v>12</v>
       </c>
       <c r="U41" s="5" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="W41" s="5" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="42">
@@ -12783,13 +12833,13 @@
         <v>0.625</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="H42" s="5" t="s">
         <v>22</v>
@@ -12798,7 +12848,7 @@
         <v>13</v>
       </c>
       <c r="J42" s="5" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -12832,227 +12882,227 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="M1" s="13" t="s">
-        <v>227</v>
+        <v>233</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="M2" s="14" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
     </row>
     <row r="5">
       <c r="M5" s="15" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="M20" s="5" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="8" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="8" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="8" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="8" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="8" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="8" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="8" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1"/>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="8" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="8" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="8" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="8" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="8" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="8" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="8" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1"/>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="8" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="8" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="8" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="8" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1"/>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="8" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="8" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="8" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="8" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="8" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="8" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
Bugle July 12, 2026
</commit_message>
<xml_diff>
--- a/Troop 79 Bugle Calendar for ICS Feed.xlsx
+++ b/Troop 79 Bugle Calendar for ICS Feed.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="822" uniqueCount="280">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="884" uniqueCount="302">
   <si>
     <t>start_date</t>
   </si>
@@ -192,18 +192,18 @@
     <t>High Adventure Trip</t>
   </si>
   <si>
+    <t>BWCA</t>
+  </si>
+  <si>
+    <t>High Adventure</t>
+  </si>
+  <si>
+    <t>02e52d7fe6a30e4623930f66937f1701@sheet2ics</t>
+  </si>
+  <si>
     <t>05ea088280e099fce97694e4f6ddf12f@sheet2ics</t>
   </si>
   <si>
-    <t>BWCA</t>
-  </si>
-  <si>
-    <t>High Adventure</t>
-  </si>
-  <si>
-    <t>02e52d7fe6a30e4623930f66937f1701@sheet2ics</t>
-  </si>
-  <si>
     <t>Camp MB Prep / Open Advancement</t>
   </si>
   <si>
@@ -216,12 +216,15 @@
     <t>290ab3dfb24f23c44b85ee236bcbf1ee@sheet2ics</t>
   </si>
   <si>
+    <t>HAT Awards, Prep for Summer Camp</t>
+  </si>
+  <si>
+    <t>38b737926b25d932e994b62a7b15a29d@sheet2ics</t>
+  </si>
+  <si>
     <t>Prep for Summer Camp</t>
   </si>
   <si>
-    <t>38b737926b25d932e994b62a7b15a29d@sheet2ics</t>
-  </si>
-  <si>
     <t>0df89d505ff7db5d0fd6917fadcafbeb@sheet2ics</t>
   </si>
   <si>
@@ -237,18 +240,51 @@
     <t>1b0cff4a338d00c5b8e27f8b9a02eac4@sheet2ics</t>
   </si>
   <si>
+    <t>Summer Camp Recovery</t>
+  </si>
+  <si>
+    <t>060b9ea3b71a8f4a8fc8ed16aa3a07b7@sheet2ics</t>
+  </si>
+  <si>
+    <t>7af7a57d8615070e2a3bdbd68b5e55d3@sheet2ics</t>
+  </si>
+  <si>
+    <t>Informal Troop Meeting - Advancement Catchup</t>
+  </si>
+  <si>
+    <t>Advancement Catchup</t>
+  </si>
+  <si>
+    <t>508827e904271d6bef65c2dd379d8fa4@sheet2ics</t>
+  </si>
+  <si>
+    <t>Rummage Sale - Prep</t>
+  </si>
+  <si>
+    <t>Rummage Sale Prep</t>
+  </si>
+  <si>
+    <t>Fund Raiser</t>
+  </si>
+  <si>
+    <t>397b25ef1c303b1b970fe870bb747dfe@sheet2ics</t>
+  </si>
+  <si>
     <t>Rummage Sale</t>
   </si>
   <si>
     <t>All Day Rummage Sale</t>
   </si>
   <si>
-    <t>Fund Raiser</t>
-  </si>
-  <si>
     <t>2a356e920aad675a7efea5fc90141738@sheet2ics</t>
   </si>
   <si>
+    <t>Labor Day</t>
+  </si>
+  <si>
+    <t>e9dd565f34016850a8c00de47d3ec6c8@sheet2ics</t>
+  </si>
+  <si>
     <t>Court of Honor - Eagle</t>
   </si>
   <si>
@@ -261,6 +297,39 @@
     <t>11a5cb096a7f6578a8ef2d5ed2b76687@sheet2ics</t>
   </si>
   <si>
+    <t>717574efc0130be9d4c58236b9e3a5ee@sheet2ics</t>
+  </si>
+  <si>
+    <t>16b9ae99d4f0ad3ad9b23e6c1f8f9a28@sheet2ics</t>
+  </si>
+  <si>
+    <t>Troop Meeting - Campout Prep</t>
+  </si>
+  <si>
+    <t>395a1a33b8520617b580ae1bd39f42a0@sheet2ics</t>
+  </si>
+  <si>
+    <t>be7814550f3b2e18e703f2c5ab47b9ac@sheet2ics</t>
+  </si>
+  <si>
+    <t>Fall Campout</t>
+  </si>
+  <si>
+    <t>TBD</t>
+  </si>
+  <si>
+    <t>f3316cb1ba683dab632173059daf4983@sheet2ics</t>
+  </si>
+  <si>
+    <t>Troop Meeting - Campout Cleanup</t>
+  </si>
+  <si>
+    <t>eb921046c8f03661cc2d7ca54e6dd34a@sheet2ics</t>
+  </si>
+  <si>
+    <t>7d34f3e0c7988225a43cd35be1c2fbae@sheet2ics</t>
+  </si>
+  <si>
     <t>timezone</t>
   </si>
   <si>
@@ -379,9 +448,6 @@
   </si>
   <si>
     <t>Annual Pancake Breakfast</t>
-  </si>
-  <si>
-    <t>TBD</t>
   </si>
   <si>
     <t>Prepare for High Adventure Trip</t>
@@ -1492,7 +1558,7 @@
         <v>0.75</v>
       </c>
       <c r="D8" s="4">
-        <v>0.2916666666678793</v>
+        <v>0.7916666666678793</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>35</v>
@@ -1736,60 +1802,60 @@
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="2">
-        <v>46194.0</v>
+        <v>46193.0</v>
       </c>
       <c r="B16" s="2">
-        <v>46194.0</v>
+        <v>46200.0</v>
       </c>
       <c r="C16" s="4">
-        <v>0.6666666666678793</v>
+        <v>0.2916666666678793</v>
       </c>
       <c r="D16" s="3">
-        <v>0.7291666666678793</v>
+        <v>0.625</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>12</v>
+        <v>58</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>18</v>
+        <v>59</v>
       </c>
       <c r="I16" s="5" t="s">
         <v>14</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="2">
-        <v>46193.0</v>
+        <v>46194.0</v>
       </c>
       <c r="B17" s="2">
-        <v>46200.0</v>
+        <v>46194.0</v>
       </c>
       <c r="C17" s="4">
-        <v>0.2916666666678793</v>
+        <v>0.6666666666678793</v>
       </c>
       <c r="D17" s="3">
-        <v>0.625</v>
+        <v>0.7291666666678793</v>
       </c>
       <c r="E17" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="F17" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="F17" s="5" t="s">
-        <v>59</v>
-      </c>
       <c r="G17" s="5" t="s">
-        <v>59</v>
+        <v>12</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="I17" s="5" t="s">
         <v>14</v>
@@ -1908,7 +1974,7 @@
         <v>18</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="G21" s="5" t="s">
         <v>12</v>
@@ -1920,7 +1986,7 @@
         <v>14</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
@@ -1937,13 +2003,13 @@
         <v>0.5416666666678793</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H22" s="5" t="s">
         <v>31</v>
@@ -1952,63 +2018,59 @@
         <v>14</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="2">
-        <v>46263.0</v>
+        <v>46236.0</v>
       </c>
       <c r="B23" s="2">
-        <v>46263.0</v>
+        <v>46236.0</v>
       </c>
       <c r="C23" s="4">
-        <v>0.375</v>
+        <v>0.6666666666678793</v>
       </c>
       <c r="D23" s="3">
-        <v>0.75</v>
+        <v>0.6770833333321207</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>73</v>
+        <v>42</v>
       </c>
       <c r="F23" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="G23" s="5" t="s">
-        <v>12</v>
-      </c>
+      <c r="G23" s="5"/>
       <c r="H23" s="5" t="s">
-        <v>75</v>
+        <v>18</v>
       </c>
       <c r="I23" s="5" t="s">
         <v>14</v>
       </c>
       <c r="J23" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="2">
-        <v>46278.0</v>
-      </c>
-      <c r="B24" s="7">
-        <v>46278.0</v>
-      </c>
-      <c r="C24" s="3">
-        <v>0.625</v>
-      </c>
-      <c r="D24" s="4">
-        <v>0.7916666666678793</v>
+        <v>46243.0</v>
+      </c>
+      <c r="B24" s="2">
+        <v>46243.0</v>
+      </c>
+      <c r="C24" s="4">
+        <v>0.6666666666678793</v>
+      </c>
+      <c r="D24" s="3">
+        <v>0.6770833333321207</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>77</v>
+        <v>42</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="G24" s="5" t="s">
-        <v>79</v>
-      </c>
+        <v>74</v>
+      </c>
+      <c r="G24" s="5"/>
       <c r="H24" s="5" t="s">
         <v>18</v>
       </c>
@@ -2016,44 +2078,369 @@
         <v>14</v>
       </c>
       <c r="J24" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="2">
+        <v>46250.0</v>
+      </c>
+      <c r="B25" s="2">
+        <v>46250.0</v>
+      </c>
+      <c r="C25" s="4">
+        <v>0.6666666666678793</v>
+      </c>
+      <c r="D25" s="3">
+        <v>0.7291666666678793</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="G25" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I25" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J25" s="5" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="26" ht="15.75" customHeight="1">
+      <c r="A26" s="2">
+        <v>46257.0</v>
+      </c>
+      <c r="B26" s="2">
+        <v>46257.0</v>
+      </c>
+      <c r="C26" s="4">
+        <v>0.6666666666678793</v>
+      </c>
+      <c r="D26" s="3">
+        <v>0.7291666666678793</v>
+      </c>
+      <c r="E26" s="5" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="25" ht="15.75" customHeight="1">
-      <c r="I25" s="8"/>
-    </row>
-    <row r="26" ht="15.75" customHeight="1">
-      <c r="I26" s="8"/>
+      <c r="F26" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="G26" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="I26" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J26" s="5" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="I27" s="8"/>
+      <c r="A27" s="2">
+        <v>46263.0</v>
+      </c>
+      <c r="B27" s="2">
+        <v>46263.0</v>
+      </c>
+      <c r="C27" s="4">
+        <v>0.375</v>
+      </c>
+      <c r="D27" s="3">
+        <v>0.75</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="G27" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H27" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="I27" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J27" s="5" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="I28" s="8"/>
+      <c r="A28" s="2">
+        <v>46271.0</v>
+      </c>
+      <c r="B28" s="2">
+        <v>46271.0</v>
+      </c>
+      <c r="C28" s="4">
+        <v>0.6666666666678793</v>
+      </c>
+      <c r="D28" s="3">
+        <v>0.6770833333321207</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="H28" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I28" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J28" s="5" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="I29" s="8"/>
+      <c r="A29" s="2">
+        <v>46278.0</v>
+      </c>
+      <c r="B29" s="7">
+        <v>46278.0</v>
+      </c>
+      <c r="C29" s="3">
+        <v>0.625</v>
+      </c>
+      <c r="D29" s="4">
+        <v>0.7916666666678793</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="G29" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="H29" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I29" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J29" s="5" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="I30" s="8"/>
+      <c r="A30" s="2">
+        <v>46285.0</v>
+      </c>
+      <c r="B30" s="2">
+        <v>46285.0</v>
+      </c>
+      <c r="C30" s="4">
+        <v>0.6666666666678793</v>
+      </c>
+      <c r="D30" s="3">
+        <v>0.7291666666678793</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G30" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H30" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I30" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J30" s="5" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="I31" s="8"/>
+      <c r="A31" s="2">
+        <v>46292.0</v>
+      </c>
+      <c r="B31" s="2">
+        <v>46292.0</v>
+      </c>
+      <c r="C31" s="4">
+        <v>0.6666666666678793</v>
+      </c>
+      <c r="D31" s="3">
+        <v>0.7291666666678793</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G31" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H31" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I31" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J31" s="5" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
-      <c r="I32" s="8"/>
+      <c r="A32" s="2">
+        <v>46299.0</v>
+      </c>
+      <c r="B32" s="2">
+        <v>46299.0</v>
+      </c>
+      <c r="C32" s="4">
+        <v>0.6666666666678793</v>
+      </c>
+      <c r="D32" s="3">
+        <v>0.7291666666678793</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="G32" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H32" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I32" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J32" s="5" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
-      <c r="I33" s="8"/>
+      <c r="A33" s="2">
+        <v>46303.0</v>
+      </c>
+      <c r="B33" s="2">
+        <v>46303.0</v>
+      </c>
+      <c r="C33" s="4">
+        <v>0.75</v>
+      </c>
+      <c r="D33" s="3">
+        <v>0.7916666666678793</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="H33" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="I33" s="5"/>
+      <c r="J33" s="5" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="I34" s="8"/>
+      <c r="A34" s="2">
+        <v>46304.0</v>
+      </c>
+      <c r="B34" s="2">
+        <v>46306.0</v>
+      </c>
+      <c r="C34" s="4">
+        <v>0.75</v>
+      </c>
+      <c r="D34" s="3">
+        <v>0.5625</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="G34" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="H34" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="I34" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J34" s="5" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
-      <c r="I35" s="8"/>
+      <c r="A35" s="2">
+        <v>46313.0</v>
+      </c>
+      <c r="B35" s="2">
+        <v>46313.0</v>
+      </c>
+      <c r="C35" s="4">
+        <v>0.6666666666678793</v>
+      </c>
+      <c r="D35" s="3">
+        <v>0.7291666666678793</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="G35" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H35" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I35" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J35" s="5" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
-      <c r="I36" s="8"/>
+      <c r="A36" s="2">
+        <v>46320.0</v>
+      </c>
+      <c r="B36" s="2">
+        <v>46320.0</v>
+      </c>
+      <c r="C36" s="4">
+        <v>0.6666666666678793</v>
+      </c>
+      <c r="D36" s="3">
+        <v>0.7291666666678793</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G36" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H36" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I36" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J36" s="5" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="I37" s="8"/>
@@ -4859,11 +5246,23 @@
     </row>
     <row r="971" ht="15.75" customHeight="1">
       <c r="I971" s="8"/>
+    </row>
+    <row r="972" ht="15.75" customHeight="1">
+      <c r="I972" s="8"/>
+    </row>
+    <row r="973" ht="15.75" customHeight="1">
+      <c r="I973" s="8"/>
+    </row>
+    <row r="974" ht="15.75" customHeight="1">
+      <c r="I974" s="8"/>
+    </row>
+    <row r="975" ht="15.75" customHeight="1">
+      <c r="I975" s="8"/>
     </row>
   </sheetData>
   <autoFilter ref="$E$1:$H$1"/>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I2:I971">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I2:I975">
       <formula1>"VEVENT,VTODO"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4920,10 +5319,10 @@
         <v>6</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>81</v>
+        <v>104</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>82</v>
+        <v>105</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>0</v>
@@ -4938,60 +5337,60 @@
         <v>3</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>83</v>
+        <v>106</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>84</v>
+        <v>107</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>85</v>
+        <v>108</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>86</v>
+        <v>109</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>87</v>
+        <v>110</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>88</v>
+        <v>111</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>89</v>
+        <v>112</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="T1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>91</v>
+        <v>114</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>92</v>
+        <v>115</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="5" t="s">
-        <v>95</v>
+        <v>118</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>96</v>
+        <v>119</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G2" s="5" t="b">
         <v>0</v>
@@ -5012,30 +5411,30 @@
         <v>18</v>
       </c>
       <c r="U2" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W2" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="5" t="s">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>102</v>
+        <v>125</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G3" s="5" t="b">
         <v>0</v>
@@ -5059,30 +5458,30 @@
         <v>18</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="5" t="s">
-        <v>104</v>
+        <v>127</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>105</v>
+        <v>128</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>106</v>
+        <v>129</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G4" s="5" t="b">
         <v>0</v>
@@ -5106,30 +5505,30 @@
         <v>18</v>
       </c>
       <c r="U4" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W4" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="5" t="s">
-        <v>107</v>
+        <v>130</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G5" s="5" t="b">
         <v>0</v>
@@ -5153,33 +5552,33 @@
         <v>13</v>
       </c>
       <c r="U5" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="V5" s="10" t="s">
-        <v>111</v>
+        <v>134</v>
       </c>
       <c r="W5" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="5" t="s">
-        <v>112</v>
+        <v>135</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>105</v>
+        <v>128</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G6" s="5" t="b">
         <v>0</v>
@@ -5200,30 +5599,30 @@
         <v>18</v>
       </c>
       <c r="U6" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W6" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="5" t="s">
-        <v>114</v>
+        <v>137</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>115</v>
+        <v>138</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>117</v>
+        <v>140</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G7" s="5" t="b">
         <v>0</v>
@@ -5247,11 +5646,11 @@
         <v>13</v>
       </c>
       <c r="U7" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="V7" s="11"/>
       <c r="W7" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
@@ -5271,7 +5670,7 @@
         <v>12</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G8" s="5" t="b">
         <v>0</v>
@@ -5295,30 +5694,30 @@
         <v>18</v>
       </c>
       <c r="U8" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W8" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="5" t="s">
-        <v>118</v>
+        <v>141</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>119</v>
+        <v>142</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>120</v>
+        <v>143</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G9" s="5" t="b">
         <v>0</v>
@@ -5339,13 +5738,13 @@
         <v>30.0</v>
       </c>
       <c r="T9" s="5" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="U9" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W9" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
@@ -5365,7 +5764,7 @@
         <v>12</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G10" s="5" t="b">
         <v>0</v>
@@ -5389,10 +5788,10 @@
         <v>18</v>
       </c>
       <c r="U10" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W10" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
@@ -5409,10 +5808,10 @@
         <v>40</v>
       </c>
       <c r="E11" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="F11" s="5" t="s">
         <v>121</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>98</v>
       </c>
       <c r="G11" s="5" t="b">
         <v>0</v>
@@ -5433,10 +5832,10 @@
         <v>31</v>
       </c>
       <c r="U11" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W11" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
@@ -5453,7 +5852,7 @@
         <v>43</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G12" s="5" t="b">
         <v>0</v>
@@ -5471,10 +5870,10 @@
         <v>0.6673611111109494</v>
       </c>
       <c r="U12" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W12" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
@@ -5488,13 +5887,13 @@
         <v>18</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>121</v>
+        <v>99</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G13" s="5" t="b">
         <v>0</v>
@@ -5518,10 +5917,10 @@
         <v>18</v>
       </c>
       <c r="U13" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W13" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
@@ -5535,13 +5934,13 @@
         <v>18</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>121</v>
+        <v>99</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G14" s="5" t="b">
         <v>0</v>
@@ -5565,10 +5964,10 @@
         <v>18</v>
       </c>
       <c r="U14" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W14" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1">
@@ -5582,13 +5981,13 @@
         <v>18</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>122</v>
+        <v>144</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G15" s="5" t="b">
         <v>0</v>
@@ -5612,15 +6011,15 @@
         <v>18</v>
       </c>
       <c r="U15" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W15" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>14</v>
@@ -5629,13 +6028,13 @@
         <v>57</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G16" s="5" t="b">
         <v>0</v>
@@ -5656,18 +6055,18 @@
         <v>30.0</v>
       </c>
       <c r="T16" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="U16" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W16" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="5" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>14</v>
@@ -5682,7 +6081,7 @@
         <v>12</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G17" s="5" t="b">
         <v>0</v>
@@ -5706,10 +6105,10 @@
         <v>18</v>
       </c>
       <c r="U17" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W17" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
@@ -5723,13 +6122,13 @@
         <v>18</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>121</v>
+        <v>99</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G18" s="5" t="b">
         <v>0</v>
@@ -5753,10 +6152,10 @@
         <v>18</v>
       </c>
       <c r="U18" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W18" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="19" ht="15.75" customHeight="1">
@@ -5773,7 +6172,7 @@
         <v>64</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G19" s="5" t="b">
         <v>0</v>
@@ -5797,10 +6196,10 @@
         <v>18</v>
       </c>
       <c r="U19" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W19" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
@@ -5814,13 +6213,13 @@
         <v>18</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>121</v>
+        <v>99</v>
       </c>
       <c r="E20" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G20" s="5" t="b">
         <v>0</v>
@@ -5844,15 +6243,15 @@
         <v>18</v>
       </c>
       <c r="U20" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W20" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>14</v>
@@ -5861,13 +6260,13 @@
         <v>18</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>121</v>
+        <v>99</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G21" s="5" t="b">
         <v>0</v>
@@ -5891,30 +6290,30 @@
         <v>18</v>
       </c>
       <c r="U21" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W21" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G22" s="5" t="b">
         <v>0</v>
@@ -5935,30 +6334,30 @@
         <v>31</v>
       </c>
       <c r="U22" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W22" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="5" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>123</v>
+        <v>145</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G23" s="5" t="b">
         <v>0</v>
@@ -5979,10 +6378,10 @@
         <v>18</v>
       </c>
       <c r="U23" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W23" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
@@ -10762,22 +11161,22 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="s">
-        <v>124</v>
+        <v>146</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>126</v>
+        <v>148</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G1" s="5" t="b">
         <v>0</v>
@@ -10795,18 +11194,18 @@
         <v>0.7708333333321207</v>
       </c>
       <c r="T1" s="5" t="s">
-        <v>127</v>
+        <v>149</v>
       </c>
       <c r="U1" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W1" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>128</v>
+        <v>150</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>14</v>
@@ -10815,13 +11214,13 @@
         <v>20</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>129</v>
+        <v>151</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G2" s="5" t="b">
         <v>0</v>
@@ -10842,30 +11241,30 @@
         <v>20</v>
       </c>
       <c r="U2" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W2" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="s">
-        <v>130</v>
+        <v>152</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>131</v>
+        <v>153</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>132</v>
+        <v>154</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>133</v>
+        <v>155</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G3" s="5" t="b">
         <v>0</v>
@@ -10886,30 +11285,30 @@
         <v>13</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="s">
-        <v>134</v>
+        <v>156</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>135</v>
+        <v>157</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>136</v>
+        <v>158</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>137</v>
+        <v>159</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G4" s="5" t="b">
         <v>0</v>
@@ -10928,18 +11327,18 @@
       </c>
       <c r="L4" s="2"/>
       <c r="T4" s="5" t="s">
-        <v>138</v>
+        <v>160</v>
       </c>
       <c r="U4" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W4" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="s">
-        <v>139</v>
+        <v>161</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>14</v>
@@ -10948,13 +11347,13 @@
         <v>20</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G5" s="5" t="b">
         <v>0</v>
@@ -10975,13 +11374,13 @@
         <v>20</v>
       </c>
       <c r="U5" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W5" s="5"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="s">
-        <v>141</v>
+        <v>163</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>14</v>
@@ -10990,13 +11389,13 @@
         <v>18</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>142</v>
+        <v>164</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G6" s="5" t="b">
         <v>0</v>
@@ -11020,30 +11419,30 @@
         <v>18</v>
       </c>
       <c r="U6" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W6" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="s">
-        <v>143</v>
+        <v>165</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>132</v>
+        <v>154</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>133</v>
+        <v>155</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G7" s="5" t="b">
         <v>0</v>
@@ -11064,30 +11463,30 @@
         <v>13</v>
       </c>
       <c r="U7" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W7" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>146</v>
+        <v>168</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>147</v>
+        <v>169</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>148</v>
+        <v>170</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G8" s="5" t="b">
         <v>0</v>
@@ -11108,18 +11507,18 @@
         <v>60.0</v>
       </c>
       <c r="T8" s="5" t="s">
-        <v>138</v>
+        <v>160</v>
       </c>
       <c r="U8" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W8" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>149</v>
+        <v>171</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>14</v>
@@ -11128,13 +11527,13 @@
         <v>18</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>150</v>
+        <v>172</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G9" s="5" t="b">
         <v>0</v>
@@ -11158,15 +11557,15 @@
         <v>18</v>
       </c>
       <c r="U9" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W9" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>151</v>
+        <v>173</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>14</v>
@@ -11175,13 +11574,13 @@
         <v>18</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>152</v>
+        <v>174</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G10" s="5" t="b">
         <v>0</v>
@@ -11205,15 +11604,15 @@
         <v>18</v>
       </c>
       <c r="U10" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W10" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="s">
-        <v>153</v>
+        <v>175</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>14</v>
@@ -11222,13 +11621,13 @@
         <v>18</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>154</v>
+        <v>176</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G11" s="5" t="b">
         <v>0</v>
@@ -11252,15 +11651,15 @@
         <v>18</v>
       </c>
       <c r="U11" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W11" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="s">
-        <v>155</v>
+        <v>177</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>14</v>
@@ -11269,13 +11668,13 @@
         <v>20</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G12" s="5" t="b">
         <v>0</v>
@@ -11296,15 +11695,15 @@
         <v>20</v>
       </c>
       <c r="U12" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W12" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="s">
-        <v>156</v>
+        <v>178</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>14</v>
@@ -11313,13 +11712,13 @@
         <v>18</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>152</v>
+        <v>174</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G13" s="5" t="b">
         <v>0</v>
@@ -11343,30 +11742,30 @@
         <v>18</v>
       </c>
       <c r="U13" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W13" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="s">
-        <v>157</v>
+        <v>179</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>158</v>
+        <v>180</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>159</v>
+        <v>181</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G14" s="5" t="b">
         <v>0</v>
@@ -11390,15 +11789,15 @@
         <v>18</v>
       </c>
       <c r="U14" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W14" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="s">
-        <v>160</v>
+        <v>182</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>14</v>
@@ -11407,10 +11806,10 @@
         <v>42</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>161</v>
+        <v>183</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G15" s="5" t="b">
         <v>0</v>
@@ -11428,15 +11827,15 @@
         <v>0.6673611111109494</v>
       </c>
       <c r="U15" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W15" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="s">
-        <v>162</v>
+        <v>184</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>14</v>
@@ -11445,10 +11844,10 @@
         <v>42</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>163</v>
+        <v>185</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G16" s="5" t="b">
         <v>0</v>
@@ -11466,15 +11865,15 @@
         <v>0.6673611111109494</v>
       </c>
       <c r="U16" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W16" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>164</v>
+        <v>186</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>14</v>
@@ -11483,13 +11882,13 @@
         <v>18</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>165</v>
+        <v>187</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G17" s="5" t="b">
         <v>0</v>
@@ -11513,15 +11912,15 @@
         <v>18</v>
       </c>
       <c r="U17" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W17" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="s">
-        <v>166</v>
+        <v>188</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>14</v>
@@ -11530,13 +11929,13 @@
         <v>20</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G18" s="5" t="b">
         <v>0</v>
@@ -11560,30 +11959,30 @@
         <v>20</v>
       </c>
       <c r="U18" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W18" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>167</v>
+        <v>189</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>168</v>
+        <v>190</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>169</v>
+        <v>191</v>
       </c>
       <c r="E19" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G19" s="5" t="b">
         <v>0</v>
@@ -11604,18 +12003,18 @@
         <v>30.0</v>
       </c>
       <c r="T19" s="5" t="s">
-        <v>170</v>
+        <v>192</v>
       </c>
       <c r="U19" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W19" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="s">
-        <v>171</v>
+        <v>193</v>
       </c>
       <c r="B20" s="5" t="s">
         <v>14</v>
@@ -11624,10 +12023,10 @@
         <v>42</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>172</v>
+        <v>194</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G20" s="5" t="b">
         <v>0</v>
@@ -11645,15 +12044,15 @@
         <v>0.6673611111109494</v>
       </c>
       <c r="U20" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W20" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="s">
-        <v>173</v>
+        <v>195</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>14</v>
@@ -11662,13 +12061,13 @@
         <v>18</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G21" s="5" t="b">
         <v>0</v>
@@ -11692,15 +12091,15 @@
         <v>18</v>
       </c>
       <c r="U21" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W21" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="s">
-        <v>174</v>
+        <v>196</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>14</v>
@@ -11709,13 +12108,13 @@
         <v>18</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="E22" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G22" s="5" t="b">
         <v>0</v>
@@ -11739,30 +12138,30 @@
         <v>18</v>
       </c>
       <c r="U22" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W22" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="5" t="s">
-        <v>175</v>
+        <v>197</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>176</v>
+        <v>198</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>177</v>
+        <v>199</v>
       </c>
       <c r="E23" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G23" s="5" t="b">
         <v>0</v>
@@ -11786,30 +12185,30 @@
         <v>18</v>
       </c>
       <c r="U23" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W23" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="5" t="s">
-        <v>178</v>
+        <v>200</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>179</v>
+        <v>201</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>180</v>
+        <v>202</v>
       </c>
       <c r="E24" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G24" s="5" t="b">
         <v>0</v>
@@ -11833,30 +12232,30 @@
         <v>18</v>
       </c>
       <c r="U24" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W24" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="5" t="s">
-        <v>181</v>
+        <v>203</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>182</v>
+        <v>204</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>183</v>
+        <v>205</v>
       </c>
       <c r="E25" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G25" s="5" t="b">
         <v>0</v>
@@ -11880,30 +12279,30 @@
         <v>18</v>
       </c>
       <c r="U25" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W25" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="5" t="s">
-        <v>184</v>
+        <v>206</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>185</v>
+        <v>207</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>186</v>
+        <v>208</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>187</v>
+        <v>209</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G26" s="5" t="b">
         <v>0</v>
@@ -11921,21 +12320,21 @@
         <v>0.6875</v>
       </c>
       <c r="T26" s="5" t="s">
-        <v>188</v>
+        <v>210</v>
       </c>
       <c r="U26" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="V26" s="12" t="s">
-        <v>189</v>
+        <v>211</v>
       </c>
       <c r="W26" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="5" t="s">
-        <v>190</v>
+        <v>212</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>14</v>
@@ -11944,13 +12343,13 @@
         <v>20</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G27" s="5" t="b">
         <v>0</v>
@@ -11971,28 +12370,28 @@
         <v>20</v>
       </c>
       <c r="U27" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W27" s="5"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="5" t="s">
-        <v>191</v>
+        <v>213</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>192</v>
+        <v>214</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>193</v>
+        <v>215</v>
       </c>
       <c r="E28" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G28" s="5" t="b">
         <v>0</v>
@@ -12010,30 +12409,30 @@
         <v>0.6736111111094942</v>
       </c>
       <c r="U28" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W28" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="5" t="s">
-        <v>194</v>
+        <v>216</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>195</v>
+        <v>217</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>195</v>
+        <v>217</v>
       </c>
       <c r="E29" s="5" t="s">
         <v>37</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G29" s="5" t="b">
         <v>0</v>
@@ -12051,33 +12450,33 @@
         <v>0.8125</v>
       </c>
       <c r="T29" s="5" t="s">
-        <v>196</v>
+        <v>218</v>
       </c>
       <c r="U29" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W29" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="5" t="s">
-        <v>197</v>
+        <v>219</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>198</v>
+        <v>220</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>198</v>
+        <v>220</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>199</v>
+        <v>221</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G30" s="5" t="b">
         <v>0</v>
@@ -12101,30 +12500,30 @@
         <v>18</v>
       </c>
       <c r="U30" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W30" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="5" t="s">
-        <v>200</v>
+        <v>222</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>201</v>
+        <v>223</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>201</v>
+        <v>223</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G31" s="5" t="b">
         <v>0</v>
@@ -12148,30 +12547,30 @@
         <v>13</v>
       </c>
       <c r="U31" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W31" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="5" t="s">
-        <v>202</v>
+        <v>224</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>203</v>
+        <v>225</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="E32" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G32" s="5" t="b">
         <v>0</v>
@@ -12195,30 +12594,30 @@
         <v>18</v>
       </c>
       <c r="U32" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W32" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="5" t="s">
-        <v>194</v>
+        <v>216</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>204</v>
+        <v>226</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>204</v>
+        <v>226</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>205</v>
+        <v>227</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G33" s="5" t="b">
         <v>0</v>
@@ -12236,33 +12635,33 @@
         <v>0.3958333333321207</v>
       </c>
       <c r="T33" s="5" t="s">
-        <v>196</v>
+        <v>218</v>
       </c>
       <c r="U33" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W33" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="5" t="s">
-        <v>206</v>
+        <v>228</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>203</v>
+        <v>225</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="E34" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G34" s="5" t="b">
         <v>0</v>
@@ -12286,30 +12685,30 @@
         <v>18</v>
       </c>
       <c r="U34" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W34" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="5" t="s">
-        <v>207</v>
+        <v>229</v>
       </c>
       <c r="B35" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>208</v>
+        <v>230</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>209</v>
+        <v>231</v>
       </c>
       <c r="E35" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G35" s="5" t="b">
         <v>0</v>
@@ -12330,33 +12729,33 @@
         <v>30.0</v>
       </c>
       <c r="T35" s="5" t="s">
-        <v>210</v>
+        <v>232</v>
       </c>
       <c r="U35" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W35" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="5" t="s">
-        <v>211</v>
+        <v>233</v>
       </c>
       <c r="B36" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>203</v>
+        <v>225</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="E36" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G36" s="5" t="b">
         <v>0</v>
@@ -12380,15 +12779,15 @@
         <v>18</v>
       </c>
       <c r="U36" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W36" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="5" t="s">
-        <v>212</v>
+        <v>234</v>
       </c>
       <c r="B37" s="5" t="s">
         <v>14</v>
@@ -12397,13 +12796,13 @@
         <v>20</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G37" s="5" t="b">
         <v>0</v>
@@ -12424,25 +12823,25 @@
         <v>20</v>
       </c>
       <c r="U37" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W37" s="5"/>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="5" t="s">
-        <v>213</v>
+        <v>235</v>
       </c>
       <c r="B38" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>214</v>
+        <v>236</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>215</v>
+        <v>237</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>216</v>
+        <v>238</v>
       </c>
       <c r="F38" s="5"/>
       <c r="G38" s="5" t="b">
@@ -12464,30 +12863,30 @@
         <v>13</v>
       </c>
       <c r="U38" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W38" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="5" t="s">
-        <v>217</v>
+        <v>239</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>203</v>
+        <v>225</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="E39" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G39" s="5" t="b">
         <v>0</v>
@@ -12511,30 +12910,30 @@
         <v>18</v>
       </c>
       <c r="U39" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W39" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="5" t="s">
-        <v>218</v>
+        <v>240</v>
       </c>
       <c r="B40" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>203</v>
+        <v>225</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>219</v>
+        <v>241</v>
       </c>
       <c r="E40" s="5" t="s">
         <v>12</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G40" s="5" t="b">
         <v>0</v>
@@ -12558,27 +12957,27 @@
         <v>18</v>
       </c>
       <c r="U40" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W40" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="5" t="s">
-        <v>220</v>
+        <v>242</v>
       </c>
       <c r="B41" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>221</v>
+        <v>243</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>222</v>
+        <v>244</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="G41" s="5" t="b">
         <v>0</v>
@@ -12599,10 +12998,10 @@
         <v>18</v>
       </c>
       <c r="U41" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="W41" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="42">
@@ -12619,13 +13018,13 @@
         <v>0.625</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>115</v>
+        <v>138</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>117</v>
+        <v>140</v>
       </c>
       <c r="H42" s="5" t="s">
         <v>13</v>
@@ -12634,7 +13033,7 @@
         <v>14</v>
       </c>
       <c r="J42" s="5" t="s">
-        <v>114</v>
+        <v>137</v>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
@@ -12651,10 +13050,10 @@
         <v>0.6875</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>96</v>
+        <v>119</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="H43" s="5" t="s">
         <v>18</v>
@@ -12663,7 +13062,7 @@
         <v>14</v>
       </c>
       <c r="J43" s="5" t="s">
-        <v>95</v>
+        <v>118</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
@@ -12680,10 +13079,10 @@
         <v>0.7291666666678793</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>102</v>
+        <v>125</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="G44" s="5" t="s">
         <v>12</v>
@@ -12695,7 +13094,7 @@
         <v>14</v>
       </c>
       <c r="J44" s="5" t="s">
-        <v>101</v>
+        <v>124</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
@@ -12712,13 +13111,13 @@
         <v>0.7916666666678793</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>223</v>
+        <v>245</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>224</v>
+        <v>246</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="H45" s="5" t="s">
         <v>13</v>
@@ -12727,7 +13126,7 @@
         <v>14</v>
       </c>
       <c r="J45" s="5" t="s">
-        <v>225</v>
+        <v>247</v>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
@@ -12744,10 +13143,10 @@
         <v>0.7291666666678793</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>226</v>
+        <v>248</v>
       </c>
       <c r="F46" s="5" t="s">
-        <v>106</v>
+        <v>129</v>
       </c>
       <c r="G46" s="5" t="s">
         <v>12</v>
@@ -12759,7 +13158,7 @@
         <v>14</v>
       </c>
       <c r="J46" s="5" t="s">
-        <v>104</v>
+        <v>127</v>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
@@ -12776,22 +13175,22 @@
         <v>0.8020833333321207</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>227</v>
+        <v>249</v>
       </c>
       <c r="F47" s="5" t="s">
-        <v>228</v>
+        <v>250</v>
       </c>
       <c r="G47" s="5" t="s">
         <v>12</v>
       </c>
       <c r="H47" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I47" s="5" t="s">
         <v>14</v>
       </c>
       <c r="J47" s="5" t="s">
-        <v>229</v>
+        <v>251</v>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1">
@@ -12808,10 +13207,10 @@
         <v>0.8125</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>230</v>
+        <v>252</v>
       </c>
       <c r="F48" s="5" t="s">
-        <v>231</v>
+        <v>253</v>
       </c>
       <c r="G48" s="5" t="s">
         <v>12</v>
@@ -12823,7 +13222,7 @@
         <v>14</v>
       </c>
       <c r="J48" s="5" t="s">
-        <v>232</v>
+        <v>254</v>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1">
@@ -12840,13 +13239,13 @@
         <v>0.6458333333321207</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="F49" s="5" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="G49" s="5" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="H49" s="5" t="s">
         <v>13</v>
@@ -12855,7 +13254,7 @@
         <v>14</v>
       </c>
       <c r="J49" s="5" t="s">
-        <v>107</v>
+        <v>130</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
@@ -12872,10 +13271,10 @@
         <v>0.7291666666678793</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>233</v>
+        <v>255</v>
       </c>
       <c r="F50" s="5" t="s">
-        <v>113</v>
+        <v>136</v>
       </c>
       <c r="G50" s="5" t="s">
         <v>12</v>
@@ -12887,7 +13286,7 @@
         <v>14</v>
       </c>
       <c r="J50" s="5" t="s">
-        <v>112</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>
@@ -12921,227 +13320,227 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>234</v>
+        <v>256</v>
       </c>
       <c r="M1" s="13" t="s">
-        <v>235</v>
+        <v>257</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="s">
-        <v>236</v>
+        <v>258</v>
       </c>
       <c r="M2" s="14" t="s">
-        <v>237</v>
+        <v>259</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="s">
-        <v>238</v>
+        <v>260</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>239</v>
+        <v>261</v>
       </c>
     </row>
     <row r="5">
       <c r="M5" s="15" t="s">
-        <v>240</v>
+        <v>262</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="s">
-        <v>241</v>
+        <v>263</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="s">
-        <v>242</v>
+        <v>264</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="s">
-        <v>243</v>
+        <v>265</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="s">
-        <v>244</v>
+        <v>266</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="s">
-        <v>245</v>
+        <v>267</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="s">
-        <v>246</v>
+        <v>268</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="s">
-        <v>247</v>
+        <v>269</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="s">
-        <v>248</v>
+        <v>270</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="s">
-        <v>249</v>
+        <v>271</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="s">
-        <v>250</v>
+        <v>272</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="s">
-        <v>251</v>
+        <v>273</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="s">
-        <v>252</v>
+        <v>274</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="s">
-        <v>253</v>
+        <v>275</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="s">
-        <v>254</v>
+        <v>276</v>
       </c>
       <c r="M20" s="5" t="s">
-        <v>255</v>
+        <v>277</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="8" t="s">
-        <v>256</v>
+        <v>278</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="8" t="s">
-        <v>257</v>
+        <v>279</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="8" t="s">
-        <v>258</v>
+        <v>280</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="8" t="s">
-        <v>259</v>
+        <v>281</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="8" t="s">
-        <v>260</v>
+        <v>282</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="8" t="s">
-        <v>261</v>
+        <v>283</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="8" t="s">
-        <v>262</v>
+        <v>284</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1"/>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="8" t="s">
-        <v>263</v>
+        <v>285</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="8" t="s">
-        <v>264</v>
+        <v>286</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="8" t="s">
-        <v>265</v>
+        <v>287</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="8" t="s">
-        <v>266</v>
+        <v>288</v>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="8" t="s">
-        <v>267</v>
+        <v>289</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="8" t="s">
-        <v>268</v>
+        <v>290</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="8" t="s">
-        <v>269</v>
+        <v>291</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1"/>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="8" t="s">
-        <v>270</v>
+        <v>292</v>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="8" t="s">
-        <v>271</v>
+        <v>293</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="8" t="s">
-        <v>272</v>
+        <v>294</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="8" t="s">
-        <v>273</v>
+        <v>295</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1"/>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="8" t="s">
-        <v>274</v>
+        <v>296</v>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="8" t="s">
-        <v>275</v>
+        <v>297</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="8" t="s">
-        <v>276</v>
+        <v>298</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="8" t="s">
-        <v>277</v>
+        <v>299</v>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="8" t="s">
-        <v>278</v>
+        <v>300</v>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="8" t="s">
-        <v>279</v>
+        <v>301</v>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1"/>

</xml_diff>